<commit_message>
Apply annual purchase volumes and add annual BOM sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjFrCobQqqs1TtLcuKd8BA
</commit_message>
<xml_diff>
--- a/IDMST_Price_List.xlsx
+++ b/IDMST_Price_List.xlsx
@@ -11,6 +11,7 @@
     <sheet name="요약" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Price List" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="기준사양 매칭" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="연간 BOM" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -266,7 +267,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="136">
   <si>
     <r>
       <rPr>
@@ -275,7 +276,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">기준사양 매칭 요약 </t>
+      <t xml:space="preserve">기준사양 매칭 요약 — 연간 구매수량 기준 </t>
     </r>
     <r>
       <rPr>
@@ -294,7 +295,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">특가 기준</t>
+      <t xml:space="preserve">특가</t>
     </r>
     <r>
       <rPr>
@@ -339,21 +340,22 @@
         <b val="true"/>
         <sz val="10"/>
         <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Set </t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 구매수량
+</t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="10"/>
         <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">수량</t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(EA)</t>
     </r>
   </si>
   <si>
@@ -458,7 +460,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">합계</t>
+      <t xml:space="preserve">연간 금액</t>
     </r>
   </si>
   <si>
@@ -491,7 +493,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">합계</t>
+      <t xml:space="preserve">연간 금액</t>
     </r>
   </si>
   <si>
@@ -524,7 +526,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">합계</t>
+      <t xml:space="preserve">연간 금액</t>
     </r>
   </si>
   <si>
@@ -581,7 +583,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">대비 차액</t>
+      <t xml:space="preserve">대비 연간 차액</t>
     </r>
   </si>
   <si>
@@ -1382,6 +1384,122 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">• 연간 구매수량</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파란 글씨</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 사용자 제공 값</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: TSU 200 / ANU 300 / ANU-S 50 / MCC 100 EA. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수량을 바꾸면 연간 금액과 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">BOM' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시트가 함께 재계산됨</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">• 파란 글씨 </t>
     </r>
     <r>
@@ -1411,26 +1529,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(Set </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF404040"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">수량 등</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF404040"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">), </t>
+      <t xml:space="preserve">, </t>
     </r>
     <r>
       <rPr>
@@ -2545,6 +2644,30 @@
   </si>
   <si>
     <t xml:space="preserve">판정</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 수량
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(EA)</t>
+    </r>
   </si>
   <si>
     <r>
@@ -3561,6 +3684,288 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">모듈별 연간 소요량 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(BOM) — </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">구성안별</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 수량 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= Σ(</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시스템별 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 set </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수량 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시스템 연간 구매수량</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수량 기반 추가 할인 협상용</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단가는 현재 특가</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">안</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">A</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">안</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">B</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">안</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">C</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">연간 수량</t>
+  </si>
+  <si>
+    <t xml:space="preserve">연간 금액</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">검증</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: '</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">요약</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">' </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 금액과 일치 여부</t>
     </r>
   </si>
 </sst>
@@ -3575,7 +3980,7 @@
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0;\-0;\-"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3732,6 +4137,19 @@
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
     </font>
+    <font>
+      <i val="true"/>
+      <sz val="9"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -3814,7 +4232,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3827,10 +4245,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3839,7 +4253,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3877,6 +4291,10 @@
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -3955,11 +4373,35 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4215,7 +4657,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -4244,7 +4686,7 @@
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="2" t="s">
@@ -4267,281 +4709,294 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="7" t="n">
+      <c r="C4" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="D4" s="6" t="n">
         <f aca="false">'기준사양 매칭'!G9</f>
         <v>457250</v>
       </c>
-      <c r="E4" s="7" t="n">
+      <c r="E4" s="6" t="n">
         <f aca="false">'기준사양 매칭'!G11</f>
         <v>392850</v>
       </c>
-      <c r="F4" s="7" t="n">
+      <c r="F4" s="6" t="n">
         <f aca="false">'기준사양 매칭'!G13</f>
         <v>384750</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="7" t="n">
         <f aca="false">$C4*D4</f>
-        <v>457250</v>
-      </c>
-      <c r="H4" s="8" t="n">
+        <v>91450000</v>
+      </c>
+      <c r="H4" s="7" t="n">
         <f aca="false">$C4*E4</f>
-        <v>392850</v>
-      </c>
-      <c r="I4" s="8" t="n">
+        <v>78570000</v>
+      </c>
+      <c r="I4" s="7" t="n">
         <f aca="false">$C4*F4</f>
-        <v>384750</v>
+        <v>76950000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="7" t="n">
+      <c r="C5" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="D5" s="6" t="n">
         <f aca="false">'기준사양 매칭'!G20</f>
         <v>622050</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="6" t="n">
         <f aca="false">'기준사양 매칭'!G23</f>
         <v>556000</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="6" t="n">
         <f aca="false">'기준사양 매칭'!G26</f>
         <v>544750</v>
       </c>
-      <c r="G5" s="8" t="n">
+      <c r="G5" s="7" t="n">
         <f aca="false">$C5*D5</f>
-        <v>622050</v>
-      </c>
-      <c r="H5" s="8" t="n">
+        <v>186615000</v>
+      </c>
+      <c r="H5" s="7" t="n">
         <f aca="false">$C5*E5</f>
-        <v>556000</v>
-      </c>
-      <c r="I5" s="8" t="n">
+        <v>166800000</v>
+      </c>
+      <c r="I5" s="7" t="n">
         <f aca="false">$C5*F5</f>
-        <v>544750</v>
+        <v>163425000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="7" t="n">
+      <c r="C6" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" s="6" t="n">
         <f aca="false">'기준사양 매칭'!G33</f>
         <v>595650</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="6" t="n">
         <f aca="false">'기준사양 매칭'!G36</f>
         <v>531250</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="6" t="n">
         <f aca="false">'기준사양 매칭'!G39</f>
         <v>523150</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="7" t="n">
         <f aca="false">$C6*D6</f>
-        <v>595650</v>
-      </c>
-      <c r="H6" s="8" t="n">
+        <v>29782500</v>
+      </c>
+      <c r="H6" s="7" t="n">
         <f aca="false">$C6*E6</f>
-        <v>531250</v>
-      </c>
-      <c r="I6" s="8" t="n">
+        <v>26562500</v>
+      </c>
+      <c r="I6" s="7" t="n">
         <f aca="false">$C6*F6</f>
-        <v>523150</v>
+        <v>26157500</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="7" t="n">
+      <c r="C7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" s="6" t="n">
         <f aca="false">'기준사양 매칭'!G47</f>
         <v>1449500</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="6" t="n">
         <f aca="false">'기준사양 매칭'!G52</f>
         <v>1358700</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F7" s="6" t="n">
         <f aca="false">'기준사양 매칭'!G57</f>
         <v>1449500</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="7" t="n">
         <f aca="false">$C7*D7</f>
-        <v>1449500</v>
-      </c>
-      <c r="H7" s="8" t="n">
+        <v>144950000</v>
+      </c>
+      <c r="H7" s="7" t="n">
         <f aca="false">$C7*E7</f>
-        <v>1358700</v>
-      </c>
-      <c r="I7" s="8" t="n">
+        <v>135870000</v>
+      </c>
+      <c r="I7" s="7" t="n">
         <f aca="false">$C7*F7</f>
-        <v>1449500</v>
+        <v>144950000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="10" t="n">
+      <c r="B8" s="8"/>
+      <c r="C8" s="9" t="n">
         <f aca="false">SUM(C4:C7)</f>
-        <v>4</v>
-      </c>
-      <c r="D8" s="11" t="n">
+        <v>650</v>
+      </c>
+      <c r="D8" s="10" t="n">
         <f aca="false">SUM(D4:D7)</f>
         <v>3124450</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="10" t="n">
         <f aca="false">SUM(E4:E7)</f>
         <v>2838800</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="10" t="n">
         <f aca="false">SUM(F4:F7)</f>
         <v>2902150</v>
       </c>
-      <c r="G8" s="11" t="n">
+      <c r="G8" s="10" t="n">
         <f aca="false">SUM(G4:G7)</f>
-        <v>3124450</v>
-      </c>
-      <c r="H8" s="11" t="n">
+        <v>452797500</v>
+      </c>
+      <c r="H8" s="10" t="n">
         <f aca="false">SUM(H4:H7)</f>
-        <v>2838800</v>
-      </c>
-      <c r="I8" s="11" t="n">
+        <v>407802500</v>
+      </c>
+      <c r="I8" s="10" t="n">
         <f aca="false">SUM(I4:I7)</f>
-        <v>2902150</v>
+        <v>411482500</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="13" t="n">
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="12" t="n">
         <f aca="false">G8-$G$8</f>
         <v>0</v>
       </c>
-      <c r="H9" s="13" t="n">
+      <c r="H9" s="12" t="n">
         <f aca="false">H8-$G$8</f>
-        <v>-285650</v>
-      </c>
-      <c r="I9" s="13" t="n">
+        <v>-44995000</v>
+      </c>
+      <c r="I9" s="12" t="n">
         <f aca="false">I8-$G$8</f>
-        <v>-222300</v>
+        <v>-41315000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
     </row>
     <row r="13" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
     </row>
     <row r="14" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
     </row>
     <row r="15" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="14"/>
     </row>
     <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="13"/>
+    </row>
+    <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A9:F9"/>
@@ -4551,6 +5006,7 @@
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A15:I15"/>
     <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A17:I17"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4587,85 +5043,85 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="B1" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="C1" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="D1" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="E1" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3" t="s">
+      <c r="F1" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3" t="s">
+      <c r="G1" s="15"/>
+      <c r="H1" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
+      <c r="Q1" s="15"/>
+      <c r="R1" s="15"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G2" s="3" t="s">
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="G2" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2" s="3" t="s">
+      <c r="H2" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="I2" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="L2" s="3" t="s">
+      <c r="J2" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="L2" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="M2" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="N2" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="O2" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="P2" s="15" t="s">
         <v>43</v>
       </c>
+      <c r="Q2" s="15" t="s">
+        <v>44</v>
+      </c>
       <c r="R2" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4673,13 +5129,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E3" s="18" t="n">
         <v>1</v>
@@ -4724,7 +5180,7 @@
         <v>1</v>
       </c>
       <c r="R3" s="17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4732,13 +5188,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E4" s="18" t="n">
         <v>1</v>
@@ -4783,7 +5239,7 @@
         <v>0</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4791,13 +5247,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E5" s="18" t="n">
         <v>1</v>
@@ -4842,7 +5298,7 @@
         <v>0</v>
       </c>
       <c r="R5" s="17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4850,13 +5306,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E6" s="18" t="n">
         <v>1</v>
@@ -4901,7 +5357,7 @@
         <v>0</v>
       </c>
       <c r="R6" s="17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4909,13 +5365,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E7" s="18" t="n">
         <v>1</v>
@@ -4960,7 +5416,7 @@
         <v>0</v>
       </c>
       <c r="R7" s="17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4968,10 +5424,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="18" t="n">
@@ -5017,7 +5473,7 @@
         <v>0</v>
       </c>
       <c r="R8" s="17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5025,10 +5481,10 @@
         <v>7</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="18" t="n">
@@ -5074,7 +5530,7 @@
         <v>0</v>
       </c>
       <c r="R9" s="17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5082,10 +5538,10 @@
         <v>8</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D10" s="16"/>
       <c r="E10" s="18" t="n">
@@ -5131,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="R10" s="17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5139,10 +5595,10 @@
         <v>9</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="18" t="n">
@@ -5188,7 +5644,7 @@
         <v>0</v>
       </c>
       <c r="R11" s="17" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5196,10 +5652,10 @@
         <v>10</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D12" s="16"/>
       <c r="E12" s="18" t="n">
@@ -5245,7 +5701,7 @@
         <v>0</v>
       </c>
       <c r="R12" s="17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5253,10 +5709,10 @@
         <v>11</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="18" t="n">
@@ -5302,7 +5758,7 @@
         <v>0</v>
       </c>
       <c r="R13" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5310,10 +5766,10 @@
         <v>12</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="18" t="n">
@@ -5359,7 +5815,7 @@
         <v>0</v>
       </c>
       <c r="R14" s="17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5367,10 +5823,10 @@
         <v>13</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D15" s="16"/>
       <c r="E15" s="18" t="n">
@@ -5416,7 +5872,7 @@
         <v>0</v>
       </c>
       <c r="R15" s="17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5424,10 +5880,10 @@
         <v>14</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D16" s="16"/>
       <c r="E16" s="18" t="n">
@@ -5473,7 +5929,7 @@
         <v>0</v>
       </c>
       <c r="R16" s="17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5481,10 +5937,10 @@
         <v>15</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D17" s="16"/>
       <c r="E17" s="18" t="n">
@@ -5530,7 +5986,7 @@
         <v>0</v>
       </c>
       <c r="R17" s="17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5538,10 +5994,10 @@
         <v>16</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D18" s="16"/>
       <c r="E18" s="18" t="n">
@@ -5587,7 +6043,7 @@
         <v>0</v>
       </c>
       <c r="R18" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5595,10 +6051,10 @@
         <v>17</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D19" s="16"/>
       <c r="E19" s="18" t="n">
@@ -5644,7 +6100,7 @@
         <v>0</v>
       </c>
       <c r="R19" s="17" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5652,10 +6108,10 @@
         <v>18</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D20" s="16"/>
       <c r="E20" s="18" t="n">
@@ -5701,22 +6157,22 @@
         <v>0</v>
       </c>
       <c r="R20" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B21" s="23"/>
       <c r="C21" s="23"/>
       <c r="D21" s="23"/>
-      <c r="E21" s="10" t="n">
+      <c r="E21" s="9" t="n">
         <f aca="false">SUM(E3:E20)</f>
         <v>18</v>
       </c>
       <c r="F21" s="24"/>
-      <c r="G21" s="11" t="n">
+      <c r="G21" s="10" t="n">
         <f aca="false">SUM(G3:G20)</f>
         <v>7662000</v>
       </c>
@@ -5725,14 +6181,14 @@
         <v>0.429006786739755</v>
       </c>
       <c r="I21" s="24"/>
-      <c r="J21" s="11" t="n">
+      <c r="J21" s="10" t="n">
         <f aca="false">SUM(J3:J20)</f>
         <v>3287050</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="26" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B23" s="26"/>
       <c r="C23" s="26"/>
@@ -5781,7 +6237,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P57"/>
+  <dimension ref="A1:Q57"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -5800,11 +6256,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5821,10 +6278,11 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="27" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -5841,60 +6299,64 @@
       <c r="N2" s="27"/>
       <c r="O2" s="27"/>
       <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>28</v>
+        <v>87</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>30</v>
+        <v>88</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>31</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I4" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="H4" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="I4" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="K4" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" s="3" t="s">
+      <c r="J4" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="K4" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="L4" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="M4" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="O4" s="3" t="s">
-        <v>91</v>
+      <c r="N4" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="O4" s="15" t="s">
+        <v>92</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B5" s="28"/>
       <c r="C5" s="28"/>
@@ -5911,17 +6373,18 @@
       <c r="N5" s="28"/>
       <c r="O5" s="28"/>
       <c r="P5" s="28"/>
+      <c r="Q5" s="28"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="29" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C6" s="30"/>
       <c r="D6" s="31" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E6" s="30"/>
       <c r="F6" s="30"/>
@@ -5945,19 +6408,20 @@
       </c>
       <c r="O6" s="30"/>
       <c r="P6" s="30"/>
+      <c r="Q6" s="30"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E7" s="33" t="n">
         <v>1</v>
@@ -6003,19 +6467,23 @@
         <v>0</v>
       </c>
       <c r="P7" s="32"/>
+      <c r="Q7" s="35" t="n">
+        <f aca="false">E7*INDEX(요약!$C$4:$C$7,MATCH($A7,요약!$A$4:$A$7,0))</f>
+        <v>200</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C8" s="32" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D8" s="32" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E8" s="33" t="n">
         <v>1</v>
@@ -6061,75 +6529,80 @@
         <v>1</v>
       </c>
       <c r="P8" s="32"/>
+      <c r="Q8" s="35" t="n">
+        <f aca="false">E8*INDEX(요약!$C$4:$C$7,MATCH($A8,요약!$A$4:$A$7,0))</f>
+        <v>200</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C9" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="D9" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="11" t="n">
+      <c r="B9" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C9" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="36" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="10" t="n">
         <f aca="false">SUM(G7:G8)</f>
         <v>457250</v>
       </c>
-      <c r="H9" s="36" t="n">
+      <c r="H9" s="37" t="n">
         <f aca="false">SUM(H7:H8)</f>
         <v>14</v>
       </c>
-      <c r="I9" s="36" t="n">
+      <c r="I9" s="37" t="n">
         <f aca="false">SUM(I7:I8)</f>
         <v>10</v>
       </c>
-      <c r="J9" s="36" t="n">
+      <c r="J9" s="37" t="n">
         <f aca="false">SUM(J7:J8)</f>
         <v>8</v>
       </c>
-      <c r="K9" s="36" t="n">
+      <c r="K9" s="37" t="n">
         <f aca="false">SUM(K7:K8)</f>
         <v>18</v>
       </c>
-      <c r="L9" s="36" t="n">
+      <c r="L9" s="37" t="n">
         <f aca="false">SUM(L7:L8)</f>
         <v>0</v>
       </c>
-      <c r="M9" s="36" t="n">
+      <c r="M9" s="37" t="n">
         <f aca="false">SUM(M7:M8)</f>
         <v>2</v>
       </c>
-      <c r="N9" s="36" t="n">
+      <c r="N9" s="37" t="n">
         <f aca="false">SUM(N7:N8)</f>
         <v>0</v>
       </c>
-      <c r="O9" s="36" t="n">
+      <c r="O9" s="37" t="n">
         <f aca="false">SUM(O7:O8)</f>
         <v>1</v>
       </c>
-      <c r="P9" s="10" t="str">
+      <c r="P9" s="9" t="str">
         <f aca="false">IF(AND(H9&gt;=H6,K9&gt;=K6,J9&gt;=K6,L9&gt;=L6,M9&gt;=M6,N9&gt;=N6),IF(O9&gt;7,"OK (TM3 버스확장 필요)","OK"),"사양 미달")</f>
         <v>OK</v>
       </c>
+      <c r="Q9" s="36"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C10" s="32" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E10" s="33" t="n">
         <v>1</v>
@@ -6175,75 +6648,80 @@
         <v>0</v>
       </c>
       <c r="P10" s="32"/>
+      <c r="Q10" s="35" t="n">
+        <f aca="false">E10*INDEX(요약!$C$4:$C$7,MATCH($A10,요약!$A$4:$A$7,0))</f>
+        <v>200</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="C11" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="D11" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="11" t="n">
+      <c r="D11" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="10" t="n">
         <f aca="false">SUM(G10:G10)</f>
         <v>392850</v>
       </c>
-      <c r="H11" s="36" t="n">
+      <c r="H11" s="37" t="n">
         <f aca="false">SUM(H10:H10)</f>
         <v>14</v>
       </c>
-      <c r="I11" s="36" t="n">
+      <c r="I11" s="37" t="n">
         <f aca="false">SUM(I10:I10)</f>
         <v>10</v>
       </c>
-      <c r="J11" s="36" t="n">
+      <c r="J11" s="37" t="n">
         <f aca="false">SUM(J10:J10)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="36" t="n">
+      <c r="K11" s="37" t="n">
         <f aca="false">SUM(K10:K10)</f>
         <v>10</v>
       </c>
-      <c r="L11" s="36" t="n">
+      <c r="L11" s="37" t="n">
         <f aca="false">SUM(L10:L10)</f>
         <v>0</v>
       </c>
-      <c r="M11" s="36" t="n">
+      <c r="M11" s="37" t="n">
         <f aca="false">SUM(M10:M10)</f>
         <v>2</v>
       </c>
-      <c r="N11" s="36" t="n">
+      <c r="N11" s="37" t="n">
         <f aca="false">SUM(N10:N10)</f>
         <v>0</v>
       </c>
-      <c r="O11" s="36" t="n">
+      <c r="O11" s="37" t="n">
         <f aca="false">SUM(O10:O10)</f>
         <v>0</v>
       </c>
-      <c r="P11" s="10" t="str">
+      <c r="P11" s="9" t="str">
         <f aca="false">IF(AND(H11&gt;=H6,K11&gt;=K6,TRUE(),L11&gt;=L6,M11&gt;=M6,N11&gt;=N6),IF(O11&gt;7,"OK (TM3 버스확장 필요)","OK"),"사양 미달")</f>
         <v>OK</v>
       </c>
+      <c r="Q11" s="36"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E12" s="33" t="n">
         <v>1</v>
@@ -6289,66 +6767,71 @@
         <v>0</v>
       </c>
       <c r="P12" s="32"/>
+      <c r="Q12" s="35" t="n">
+        <f aca="false">E12*INDEX(요약!$C$4:$C$7,MATCH($A12,요약!$A$4:$A$7,0))</f>
+        <v>200</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="C13" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="D13" s="35" t="s">
+      <c r="B13" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="11" t="n">
+      <c r="C13" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13" s="36" t="s">
+        <v>108</v>
+      </c>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="10" t="n">
         <f aca="false">SUM(G12:G12)</f>
         <v>384750</v>
       </c>
-      <c r="H13" s="36" t="n">
+      <c r="H13" s="37" t="n">
         <f aca="false">SUM(H12:H12)</f>
         <v>14</v>
       </c>
-      <c r="I13" s="36" t="n">
+      <c r="I13" s="37" t="n">
         <f aca="false">SUM(I12:I12)</f>
         <v>4</v>
       </c>
-      <c r="J13" s="36" t="n">
+      <c r="J13" s="37" t="n">
         <f aca="false">SUM(J12:J12)</f>
         <v>6</v>
       </c>
-      <c r="K13" s="36" t="n">
+      <c r="K13" s="37" t="n">
         <f aca="false">SUM(K12:K12)</f>
         <v>10</v>
       </c>
-      <c r="L13" s="36" t="n">
+      <c r="L13" s="37" t="n">
         <f aca="false">SUM(L12:L12)</f>
         <v>0</v>
       </c>
-      <c r="M13" s="36" t="n">
+      <c r="M13" s="37" t="n">
         <f aca="false">SUM(M12:M12)</f>
         <v>2</v>
       </c>
-      <c r="N13" s="36" t="n">
+      <c r="N13" s="37" t="n">
         <f aca="false">SUM(N12:N12)</f>
         <v>0</v>
       </c>
-      <c r="O13" s="36" t="n">
+      <c r="O13" s="37" t="n">
         <f aca="false">SUM(O12:O12)</f>
         <v>0</v>
       </c>
-      <c r="P13" s="10" t="str">
+      <c r="P13" s="9" t="str">
         <f aca="false">IF(AND(H13&gt;=H6,K13&gt;=K6,J13&gt;=K6,L13&gt;=L6,M13&gt;=M6,N13&gt;=N6),IF(O13&gt;7,"OK (TM3 버스확장 필요)","OK"),"사양 미달")</f>
         <v>OK</v>
       </c>
+      <c r="Q13" s="36"/>
     </row>
     <row r="15" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B15" s="28"/>
       <c r="C15" s="28"/>
@@ -6365,17 +6848,18 @@
       <c r="N15" s="28"/>
       <c r="O15" s="28"/>
       <c r="P15" s="28"/>
+      <c r="Q15" s="28"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="29" t="s">
         <v>12</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C16" s="30"/>
       <c r="D16" s="31" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E16" s="30"/>
       <c r="F16" s="30"/>
@@ -6399,19 +6883,20 @@
       </c>
       <c r="O16" s="30"/>
       <c r="P16" s="30"/>
+      <c r="Q16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
         <v>12</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C17" s="32" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E17" s="33" t="n">
         <v>1</v>
@@ -6457,19 +6942,23 @@
         <v>0</v>
       </c>
       <c r="P17" s="32"/>
+      <c r="Q17" s="35" t="n">
+        <f aca="false">E17*INDEX(요약!$C$4:$C$7,MATCH($A17,요약!$A$4:$A$7,0))</f>
+        <v>300</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
         <v>12</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C18" s="32" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E18" s="33" t="n">
         <v>1</v>
@@ -6515,19 +7004,23 @@
         <v>1</v>
       </c>
       <c r="P18" s="32"/>
+      <c r="Q18" s="35" t="n">
+        <f aca="false">E18*INDEX(요약!$C$4:$C$7,MATCH($A18,요약!$A$4:$A$7,0))</f>
+        <v>300</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
         <v>12</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C19" s="32" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E19" s="33" t="n">
         <v>1</v>
@@ -6573,75 +7066,80 @@
         <v>1</v>
       </c>
       <c r="P19" s="32"/>
+      <c r="Q19" s="35" t="n">
+        <f aca="false">E19*INDEX(요약!$C$4:$C$7,MATCH($A19,요약!$A$4:$A$7,0))</f>
+        <v>300</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C20" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="D20" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35"/>
-      <c r="G20" s="11" t="n">
+      <c r="B20" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C20" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="D20" s="36" t="s">
+        <v>102</v>
+      </c>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="10" t="n">
         <f aca="false">SUM(G17:G19)</f>
         <v>622050</v>
       </c>
-      <c r="H20" s="36" t="n">
+      <c r="H20" s="37" t="n">
         <f aca="false">SUM(H17:H19)</f>
         <v>14</v>
       </c>
-      <c r="I20" s="36" t="n">
+      <c r="I20" s="37" t="n">
         <f aca="false">SUM(I17:I19)</f>
         <v>10</v>
       </c>
-      <c r="J20" s="36" t="n">
+      <c r="J20" s="37" t="n">
         <f aca="false">SUM(J17:J19)</f>
         <v>16</v>
       </c>
-      <c r="K20" s="36" t="n">
+      <c r="K20" s="37" t="n">
         <f aca="false">SUM(K17:K19)</f>
         <v>26</v>
       </c>
-      <c r="L20" s="36" t="n">
+      <c r="L20" s="37" t="n">
         <f aca="false">SUM(L17:L19)</f>
         <v>2</v>
       </c>
-      <c r="M20" s="36" t="n">
+      <c r="M20" s="37" t="n">
         <f aca="false">SUM(M17:M19)</f>
         <v>2</v>
       </c>
-      <c r="N20" s="36" t="n">
+      <c r="N20" s="37" t="n">
         <f aca="false">SUM(N17:N19)</f>
         <v>0</v>
       </c>
-      <c r="O20" s="36" t="n">
+      <c r="O20" s="37" t="n">
         <f aca="false">SUM(O17:O19)</f>
         <v>2</v>
       </c>
-      <c r="P20" s="10" t="str">
+      <c r="P20" s="9" t="str">
         <f aca="false">IF(AND(H20&gt;=H16,K20&gt;=K16,J20&gt;=K16,L20&gt;=L16,M20&gt;=M16,N20&gt;=N16),IF(O20&gt;7,"OK (TM3 버스확장 필요)","OK"),"사양 미달")</f>
         <v>OK</v>
       </c>
+      <c r="Q20" s="36"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
         <v>12</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C21" s="32" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D21" s="32" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E21" s="33" t="n">
         <v>1</v>
@@ -6687,19 +7185,23 @@
         <v>0</v>
       </c>
       <c r="P21" s="32"/>
+      <c r="Q21" s="35" t="n">
+        <f aca="false">E21*INDEX(요약!$C$4:$C$7,MATCH($A21,요약!$A$4:$A$7,0))</f>
+        <v>300</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
         <v>12</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C22" s="32" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D22" s="32" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E22" s="33" t="n">
         <v>1</v>
@@ -6745,75 +7247,80 @@
         <v>1</v>
       </c>
       <c r="P22" s="32"/>
+      <c r="Q22" s="35" t="n">
+        <f aca="false">E22*INDEX(요약!$C$4:$C$7,MATCH($A22,요약!$A$4:$A$7,0))</f>
+        <v>300</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C23" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="C23" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="D23" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35"/>
-      <c r="G23" s="11" t="n">
+      <c r="D23" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="E23" s="36"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="10" t="n">
         <f aca="false">SUM(G21:G22)</f>
         <v>556000</v>
       </c>
-      <c r="H23" s="36" t="n">
+      <c r="H23" s="37" t="n">
         <f aca="false">SUM(H21:H22)</f>
         <v>24</v>
       </c>
-      <c r="I23" s="36" t="n">
+      <c r="I23" s="37" t="n">
         <f aca="false">SUM(I21:I22)</f>
         <v>16</v>
       </c>
-      <c r="J23" s="36" t="n">
+      <c r="J23" s="37" t="n">
         <f aca="false">SUM(J21:J22)</f>
         <v>0</v>
       </c>
-      <c r="K23" s="36" t="n">
+      <c r="K23" s="37" t="n">
         <f aca="false">SUM(K21:K22)</f>
         <v>16</v>
       </c>
-      <c r="L23" s="36" t="n">
+      <c r="L23" s="37" t="n">
         <f aca="false">SUM(L21:L22)</f>
         <v>2</v>
       </c>
-      <c r="M23" s="36" t="n">
+      <c r="M23" s="37" t="n">
         <f aca="false">SUM(M21:M22)</f>
         <v>2</v>
       </c>
-      <c r="N23" s="36" t="n">
+      <c r="N23" s="37" t="n">
         <f aca="false">SUM(N21:N22)</f>
         <v>0</v>
       </c>
-      <c r="O23" s="36" t="n">
+      <c r="O23" s="37" t="n">
         <f aca="false">SUM(O21:O22)</f>
         <v>1</v>
       </c>
-      <c r="P23" s="10" t="str">
+      <c r="P23" s="9" t="str">
         <f aca="false">IF(AND(H23&gt;=H16,K23&gt;=K16,TRUE(),L23&gt;=L16,M23&gt;=M16,N23&gt;=N16),IF(O23&gt;7,"OK (TM3 버스확장 필요)","OK"),"사양 미달")</f>
         <v>OK</v>
       </c>
+      <c r="Q23" s="36"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="s">
         <v>12</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C24" s="32" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D24" s="32" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E24" s="33" t="n">
         <v>1</v>
@@ -6859,19 +7366,23 @@
         <v>0</v>
       </c>
       <c r="P24" s="32"/>
+      <c r="Q24" s="35" t="n">
+        <f aca="false">E24*INDEX(요약!$C$4:$C$7,MATCH($A24,요약!$A$4:$A$7,0))</f>
+        <v>300</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16" t="s">
         <v>12</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C25" s="32" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D25" s="32" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E25" s="33" t="n">
         <v>1</v>
@@ -6917,66 +7428,71 @@
         <v>1</v>
       </c>
       <c r="P25" s="32"/>
+      <c r="Q25" s="35" t="n">
+        <f aca="false">E25*INDEX(요약!$C$4:$C$7,MATCH($A25,요약!$A$4:$A$7,0))</f>
+        <v>300</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B26" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="C26" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="D26" s="35" t="s">
+      <c r="B26" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="E26" s="35"/>
-      <c r="F26" s="35"/>
-      <c r="G26" s="11" t="n">
+      <c r="C26" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="D26" s="36" t="s">
+        <v>108</v>
+      </c>
+      <c r="E26" s="36"/>
+      <c r="F26" s="36"/>
+      <c r="G26" s="10" t="n">
         <f aca="false">SUM(G24:G25)</f>
         <v>544750</v>
       </c>
-      <c r="H26" s="36" t="n">
+      <c r="H26" s="37" t="n">
         <f aca="false">SUM(H24:H25)</f>
         <v>24</v>
       </c>
-      <c r="I26" s="36" t="n">
+      <c r="I26" s="37" t="n">
         <f aca="false">SUM(I24:I25)</f>
         <v>4</v>
       </c>
-      <c r="J26" s="36" t="n">
+      <c r="J26" s="37" t="n">
         <f aca="false">SUM(J24:J25)</f>
         <v>12</v>
       </c>
-      <c r="K26" s="36" t="n">
+      <c r="K26" s="37" t="n">
         <f aca="false">SUM(K24:K25)</f>
         <v>16</v>
       </c>
-      <c r="L26" s="36" t="n">
+      <c r="L26" s="37" t="n">
         <f aca="false">SUM(L24:L25)</f>
         <v>2</v>
       </c>
-      <c r="M26" s="36" t="n">
+      <c r="M26" s="37" t="n">
         <f aca="false">SUM(M24:M25)</f>
         <v>2</v>
       </c>
-      <c r="N26" s="36" t="n">
+      <c r="N26" s="37" t="n">
         <f aca="false">SUM(N24:N25)</f>
         <v>0</v>
       </c>
-      <c r="O26" s="36" t="n">
+      <c r="O26" s="37" t="n">
         <f aca="false">SUM(O24:O25)</f>
         <v>1</v>
       </c>
-      <c r="P26" s="10" t="str">
+      <c r="P26" s="9" t="str">
         <f aca="false">IF(AND(H26&gt;=H16,K26&gt;=K16,J26&gt;=K16,L26&gt;=L16,M26&gt;=M16,N26&gt;=N16),IF(O26&gt;7,"OK (TM3 버스확장 필요)","OK"),"사양 미달")</f>
         <v>OK</v>
       </c>
+      <c r="Q26" s="36"/>
     </row>
     <row r="28" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="28" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B28" s="28"/>
       <c r="C28" s="28"/>
@@ -6993,17 +7509,18 @@
       <c r="N28" s="28"/>
       <c r="O28" s="28"/>
       <c r="P28" s="28"/>
+      <c r="Q28" s="28"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="29" t="s">
         <v>14</v>
       </c>
       <c r="B29" s="30" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C29" s="30"/>
       <c r="D29" s="31" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E29" s="30"/>
       <c r="F29" s="30"/>
@@ -7027,19 +7544,20 @@
       </c>
       <c r="O29" s="30"/>
       <c r="P29" s="30"/>
+      <c r="Q29" s="30"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C30" s="32" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D30" s="32" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E30" s="33" t="n">
         <v>1</v>
@@ -7085,19 +7603,23 @@
         <v>0</v>
       </c>
       <c r="P30" s="32"/>
+      <c r="Q30" s="35" t="n">
+        <f aca="false">E30*INDEX(요약!$C$4:$C$7,MATCH($A30,요약!$A$4:$A$7,0))</f>
+        <v>50</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C31" s="32" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D31" s="32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E31" s="33" t="n">
         <v>1</v>
@@ -7143,19 +7665,23 @@
         <v>1</v>
       </c>
       <c r="P31" s="32"/>
+      <c r="Q31" s="35" t="n">
+        <f aca="false">E31*INDEX(요약!$C$4:$C$7,MATCH($A31,요약!$A$4:$A$7,0))</f>
+        <v>50</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C32" s="32" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D32" s="32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E32" s="33" t="n">
         <v>1</v>
@@ -7201,75 +7727,80 @@
         <v>1</v>
       </c>
       <c r="P32" s="32"/>
+      <c r="Q32" s="35" t="n">
+        <f aca="false">E32*INDEX(요약!$C$4:$C$7,MATCH($A32,요약!$A$4:$A$7,0))</f>
+        <v>50</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10" t="s">
+      <c r="A33" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B33" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C33" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="D33" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="E33" s="35"/>
-      <c r="F33" s="35"/>
-      <c r="G33" s="11" t="n">
+      <c r="B33" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C33" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="D33" s="36" t="s">
+        <v>102</v>
+      </c>
+      <c r="E33" s="36"/>
+      <c r="F33" s="36"/>
+      <c r="G33" s="10" t="n">
         <f aca="false">SUM(G30:G32)</f>
         <v>595650</v>
       </c>
-      <c r="H33" s="36" t="n">
+      <c r="H33" s="37" t="n">
         <f aca="false">SUM(H30:H32)</f>
         <v>14</v>
       </c>
-      <c r="I33" s="36" t="n">
+      <c r="I33" s="37" t="n">
         <f aca="false">SUM(I30:I32)</f>
         <v>10</v>
       </c>
-      <c r="J33" s="36" t="n">
+      <c r="J33" s="37" t="n">
         <f aca="false">SUM(J30:J32)</f>
         <v>8</v>
       </c>
-      <c r="K33" s="36" t="n">
+      <c r="K33" s="37" t="n">
         <f aca="false">SUM(K30:K32)</f>
         <v>18</v>
       </c>
-      <c r="L33" s="36" t="n">
+      <c r="L33" s="37" t="n">
         <f aca="false">SUM(L30:L32)</f>
         <v>2</v>
       </c>
-      <c r="M33" s="36" t="n">
+      <c r="M33" s="37" t="n">
         <f aca="false">SUM(M30:M32)</f>
         <v>2</v>
       </c>
-      <c r="N33" s="36" t="n">
+      <c r="N33" s="37" t="n">
         <f aca="false">SUM(N30:N32)</f>
         <v>0</v>
       </c>
-      <c r="O33" s="36" t="n">
+      <c r="O33" s="37" t="n">
         <f aca="false">SUM(O30:O32)</f>
         <v>2</v>
       </c>
-      <c r="P33" s="10" t="str">
+      <c r="P33" s="9" t="str">
         <f aca="false">IF(AND(H33&gt;=H29,K33&gt;=K29,J33&gt;=K29,L33&gt;=L29,M33&gt;=M29,N33&gt;=N29),IF(O33&gt;7,"OK (TM3 버스확장 필요)","OK"),"사양 미달")</f>
         <v>OK</v>
       </c>
+      <c r="Q33" s="36"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C34" s="32" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D34" s="32" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E34" s="33" t="n">
         <v>1</v>
@@ -7315,19 +7846,23 @@
         <v>0</v>
       </c>
       <c r="P34" s="32"/>
+      <c r="Q34" s="35" t="n">
+        <f aca="false">E34*INDEX(요약!$C$4:$C$7,MATCH($A34,요약!$A$4:$A$7,0))</f>
+        <v>50</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C35" s="32" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D35" s="32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E35" s="33" t="n">
         <v>1</v>
@@ -7373,75 +7908,80 @@
         <v>1</v>
       </c>
       <c r="P35" s="32"/>
+      <c r="Q35" s="35" t="n">
+        <f aca="false">E35*INDEX(요약!$C$4:$C$7,MATCH($A35,요약!$A$4:$A$7,0))</f>
+        <v>50</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="10" t="s">
+      <c r="A36" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B36" s="10" t="s">
+      <c r="B36" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C36" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="C36" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="D36" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="E36" s="35"/>
-      <c r="F36" s="35"/>
-      <c r="G36" s="11" t="n">
+      <c r="D36" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="E36" s="36"/>
+      <c r="F36" s="36"/>
+      <c r="G36" s="10" t="n">
         <f aca="false">SUM(G34:G35)</f>
         <v>531250</v>
       </c>
-      <c r="H36" s="36" t="n">
+      <c r="H36" s="37" t="n">
         <f aca="false">SUM(H34:H35)</f>
         <v>14</v>
       </c>
-      <c r="I36" s="36" t="n">
+      <c r="I36" s="37" t="n">
         <f aca="false">SUM(I34:I35)</f>
         <v>10</v>
       </c>
-      <c r="J36" s="36" t="n">
+      <c r="J36" s="37" t="n">
         <f aca="false">SUM(J34:J35)</f>
         <v>0</v>
       </c>
-      <c r="K36" s="36" t="n">
+      <c r="K36" s="37" t="n">
         <f aca="false">SUM(K34:K35)</f>
         <v>10</v>
       </c>
-      <c r="L36" s="36" t="n">
+      <c r="L36" s="37" t="n">
         <f aca="false">SUM(L34:L35)</f>
         <v>2</v>
       </c>
-      <c r="M36" s="36" t="n">
+      <c r="M36" s="37" t="n">
         <f aca="false">SUM(M34:M35)</f>
         <v>2</v>
       </c>
-      <c r="N36" s="36" t="n">
+      <c r="N36" s="37" t="n">
         <f aca="false">SUM(N34:N35)</f>
         <v>0</v>
       </c>
-      <c r="O36" s="36" t="n">
+      <c r="O36" s="37" t="n">
         <f aca="false">SUM(O34:O35)</f>
         <v>1</v>
       </c>
-      <c r="P36" s="10" t="str">
+      <c r="P36" s="9" t="str">
         <f aca="false">IF(AND(H36&gt;=H29,K36&gt;=K29,TRUE(),L36&gt;=L29,M36&gt;=M29,N36&gt;=N29),IF(O36&gt;7,"OK (TM3 버스확장 필요)","OK"),"사양 미달")</f>
         <v>OK</v>
       </c>
+      <c r="Q36" s="36"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C37" s="32" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D37" s="32" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E37" s="33" t="n">
         <v>1</v>
@@ -7487,19 +8027,23 @@
         <v>0</v>
       </c>
       <c r="P37" s="32"/>
+      <c r="Q37" s="35" t="n">
+        <f aca="false">E37*INDEX(요약!$C$4:$C$7,MATCH($A37,요약!$A$4:$A$7,0))</f>
+        <v>50</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C38" s="32" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D38" s="32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E38" s="33" t="n">
         <v>1</v>
@@ -7545,66 +8089,71 @@
         <v>1</v>
       </c>
       <c r="P38" s="32"/>
+      <c r="Q38" s="35" t="n">
+        <f aca="false">E38*INDEX(요약!$C$4:$C$7,MATCH($A38,요약!$A$4:$A$7,0))</f>
+        <v>50</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="10" t="s">
+      <c r="A39" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B39" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="C39" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="D39" s="35" t="s">
+      <c r="B39" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="E39" s="35"/>
-      <c r="F39" s="35"/>
-      <c r="G39" s="11" t="n">
+      <c r="C39" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="D39" s="36" t="s">
+        <v>108</v>
+      </c>
+      <c r="E39" s="36"/>
+      <c r="F39" s="36"/>
+      <c r="G39" s="10" t="n">
         <f aca="false">SUM(G37:G38)</f>
         <v>523150</v>
       </c>
-      <c r="H39" s="36" t="n">
+      <c r="H39" s="37" t="n">
         <f aca="false">SUM(H37:H38)</f>
         <v>14</v>
       </c>
-      <c r="I39" s="36" t="n">
+      <c r="I39" s="37" t="n">
         <f aca="false">SUM(I37:I38)</f>
         <v>4</v>
       </c>
-      <c r="J39" s="36" t="n">
+      <c r="J39" s="37" t="n">
         <f aca="false">SUM(J37:J38)</f>
         <v>6</v>
       </c>
-      <c r="K39" s="36" t="n">
+      <c r="K39" s="37" t="n">
         <f aca="false">SUM(K37:K38)</f>
         <v>10</v>
       </c>
-      <c r="L39" s="36" t="n">
+      <c r="L39" s="37" t="n">
         <f aca="false">SUM(L37:L38)</f>
         <v>2</v>
       </c>
-      <c r="M39" s="36" t="n">
+      <c r="M39" s="37" t="n">
         <f aca="false">SUM(M37:M38)</f>
         <v>2</v>
       </c>
-      <c r="N39" s="36" t="n">
+      <c r="N39" s="37" t="n">
         <f aca="false">SUM(N37:N38)</f>
         <v>0</v>
       </c>
-      <c r="O39" s="36" t="n">
+      <c r="O39" s="37" t="n">
         <f aca="false">SUM(O37:O38)</f>
         <v>1</v>
       </c>
-      <c r="P39" s="10" t="str">
+      <c r="P39" s="9" t="str">
         <f aca="false">IF(AND(H39&gt;=H29,K39&gt;=K29,J39&gt;=K29,L39&gt;=L29,M39&gt;=M29,N39&gt;=N29),IF(O39&gt;7,"OK (TM3 버스확장 필요)","OK"),"사양 미달")</f>
         <v>OK</v>
       </c>
+      <c r="Q39" s="36"/>
     </row>
     <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="28" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B41" s="28"/>
       <c r="C41" s="28"/>
@@ -7621,17 +8170,18 @@
       <c r="N41" s="28"/>
       <c r="O41" s="28"/>
       <c r="P41" s="28"/>
+      <c r="Q41" s="28"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="29" t="s">
         <v>16</v>
       </c>
       <c r="B42" s="30" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C42" s="30"/>
       <c r="D42" s="31" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E42" s="30"/>
       <c r="F42" s="30"/>
@@ -7655,19 +8205,20 @@
       </c>
       <c r="O42" s="30"/>
       <c r="P42" s="30"/>
+      <c r="Q42" s="30"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C43" s="32" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D43" s="32" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E43" s="33" t="n">
         <v>1</v>
@@ -7713,19 +8264,23 @@
         <v>0</v>
       </c>
       <c r="P43" s="32"/>
+      <c r="Q43" s="35" t="n">
+        <f aca="false">E43*INDEX(요약!$C$4:$C$7,MATCH($A43,요약!$A$4:$A$7,0))</f>
+        <v>100</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C44" s="32" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D44" s="32" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E44" s="33" t="n">
         <v>6</v>
@@ -7771,19 +8326,23 @@
         <v>6</v>
       </c>
       <c r="P44" s="32"/>
+      <c r="Q44" s="35" t="n">
+        <f aca="false">E44*INDEX(요약!$C$4:$C$7,MATCH($A44,요약!$A$4:$A$7,0))</f>
+        <v>600</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C45" s="32" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D45" s="32" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E45" s="33" t="n">
         <v>4</v>
@@ -7829,19 +8388,23 @@
         <v>4</v>
       </c>
       <c r="P45" s="32"/>
+      <c r="Q45" s="35" t="n">
+        <f aca="false">E45*INDEX(요약!$C$4:$C$7,MATCH($A45,요약!$A$4:$A$7,0))</f>
+        <v>400</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B46" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C46" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D46" s="32" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E46" s="33" t="n">
         <v>1</v>
@@ -7887,75 +8450,80 @@
         <v>1</v>
       </c>
       <c r="P46" s="32"/>
+      <c r="Q46" s="35" t="n">
+        <f aca="false">E46*INDEX(요약!$C$4:$C$7,MATCH($A46,요약!$A$4:$A$7,0))</f>
+        <v>100</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="10" t="s">
+      <c r="A47" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B47" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C47" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="D47" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="E47" s="35"/>
-      <c r="F47" s="35"/>
-      <c r="G47" s="11" t="n">
+      <c r="B47" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C47" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="D47" s="36" t="s">
+        <v>102</v>
+      </c>
+      <c r="E47" s="36"/>
+      <c r="F47" s="36"/>
+      <c r="G47" s="10" t="n">
         <f aca="false">SUM(G43:G46)</f>
         <v>1449500</v>
       </c>
-      <c r="H47" s="36" t="n">
+      <c r="H47" s="37" t="n">
         <f aca="false">SUM(H43:H46)</f>
         <v>110</v>
       </c>
-      <c r="I47" s="36" t="n">
+      <c r="I47" s="37" t="n">
         <f aca="false">SUM(I43:I46)</f>
         <v>10</v>
       </c>
-      <c r="J47" s="36" t="n">
+      <c r="J47" s="37" t="n">
         <f aca="false">SUM(J43:J46)</f>
         <v>64</v>
       </c>
-      <c r="K47" s="36" t="n">
+      <c r="K47" s="37" t="n">
         <f aca="false">SUM(K43:K46)</f>
         <v>74</v>
       </c>
-      <c r="L47" s="36" t="n">
+      <c r="L47" s="37" t="n">
         <f aca="false">SUM(L43:L46)</f>
         <v>4</v>
       </c>
-      <c r="M47" s="36" t="n">
+      <c r="M47" s="37" t="n">
         <f aca="false">SUM(M43:M46)</f>
         <v>2</v>
       </c>
-      <c r="N47" s="36" t="n">
+      <c r="N47" s="37" t="n">
         <f aca="false">SUM(N43:N46)</f>
         <v>1</v>
       </c>
-      <c r="O47" s="36" t="n">
+      <c r="O47" s="37" t="n">
         <f aca="false">SUM(O43:O46)</f>
         <v>11</v>
       </c>
-      <c r="P47" s="10" t="str">
+      <c r="P47" s="9" t="str">
         <f aca="false">IF(AND(H47&gt;=H42,K47&gt;=K42,J47&gt;=K42,L47&gt;=L42,M47&gt;=M42,N47&gt;=N42),IF(O47&gt;7,"OK (TM3 버스확장 필요)","OK"),"사양 미달")</f>
         <v>OK (TM3 버스확장 필요)</v>
       </c>
+      <c r="Q47" s="36"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C48" s="32" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D48" s="32" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E48" s="33" t="n">
         <v>1</v>
@@ -8001,19 +8569,23 @@
         <v>0</v>
       </c>
       <c r="P48" s="32"/>
+      <c r="Q48" s="35" t="n">
+        <f aca="false">E48*INDEX(요약!$C$4:$C$7,MATCH($A48,요약!$A$4:$A$7,0))</f>
+        <v>100</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C49" s="32" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D49" s="32" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E49" s="33" t="n">
         <v>6</v>
@@ -8059,19 +8631,23 @@
         <v>6</v>
       </c>
       <c r="P49" s="32"/>
+      <c r="Q49" s="35" t="n">
+        <f aca="false">E49*INDEX(요약!$C$4:$C$7,MATCH($A49,요약!$A$4:$A$7,0))</f>
+        <v>600</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B50" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C50" s="32" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D50" s="32" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E50" s="33" t="n">
         <v>3</v>
@@ -8117,19 +8693,23 @@
         <v>3</v>
       </c>
       <c r="P50" s="32"/>
+      <c r="Q50" s="35" t="n">
+        <f aca="false">E50*INDEX(요약!$C$4:$C$7,MATCH($A50,요약!$A$4:$A$7,0))</f>
+        <v>300</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B51" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C51" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D51" s="32" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E51" s="33" t="n">
         <v>1</v>
@@ -8175,75 +8755,80 @@
         <v>1</v>
       </c>
       <c r="P51" s="32"/>
+      <c r="Q51" s="35" t="n">
+        <f aca="false">E51*INDEX(요약!$C$4:$C$7,MATCH($A51,요약!$A$4:$A$7,0))</f>
+        <v>100</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="10" t="s">
+      <c r="A52" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B52" s="10" t="s">
+      <c r="B52" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C52" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="C52" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="D52" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="E52" s="35"/>
-      <c r="F52" s="35"/>
-      <c r="G52" s="11" t="n">
+      <c r="D52" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="E52" s="36"/>
+      <c r="F52" s="36"/>
+      <c r="G52" s="10" t="n">
         <f aca="false">SUM(G48:G51)</f>
         <v>1358700</v>
       </c>
-      <c r="H52" s="36" t="n">
+      <c r="H52" s="37" t="n">
         <f aca="false">SUM(H48:H51)</f>
         <v>110</v>
       </c>
-      <c r="I52" s="36" t="n">
+      <c r="I52" s="37" t="n">
         <f aca="false">SUM(I48:I51)</f>
         <v>58</v>
       </c>
-      <c r="J52" s="36" t="n">
+      <c r="J52" s="37" t="n">
         <f aca="false">SUM(J48:J51)</f>
         <v>0</v>
       </c>
-      <c r="K52" s="36" t="n">
+      <c r="K52" s="37" t="n">
         <f aca="false">SUM(K48:K51)</f>
         <v>58</v>
       </c>
-      <c r="L52" s="36" t="n">
+      <c r="L52" s="37" t="n">
         <f aca="false">SUM(L48:L51)</f>
         <v>4</v>
       </c>
-      <c r="M52" s="36" t="n">
+      <c r="M52" s="37" t="n">
         <f aca="false">SUM(M48:M51)</f>
         <v>2</v>
       </c>
-      <c r="N52" s="36" t="n">
+      <c r="N52" s="37" t="n">
         <f aca="false">SUM(N48:N51)</f>
         <v>1</v>
       </c>
-      <c r="O52" s="36" t="n">
+      <c r="O52" s="37" t="n">
         <f aca="false">SUM(O48:O51)</f>
         <v>10</v>
       </c>
-      <c r="P52" s="10" t="str">
+      <c r="P52" s="9" t="str">
         <f aca="false">IF(AND(H52&gt;=H42,K52&gt;=K42,TRUE(),L52&gt;=L42,M52&gt;=M42,N52&gt;=N42),IF(O52&gt;7,"OK (TM3 버스확장 필요)","OK"),"사양 미달")</f>
         <v>OK (TM3 버스확장 필요)</v>
       </c>
+      <c r="Q52" s="36"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B53" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C53" s="32" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D53" s="32" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E53" s="33" t="n">
         <v>1</v>
@@ -8289,19 +8874,23 @@
         <v>0</v>
       </c>
       <c r="P53" s="32"/>
+      <c r="Q53" s="35" t="n">
+        <f aca="false">E53*INDEX(요약!$C$4:$C$7,MATCH($A53,요약!$A$4:$A$7,0))</f>
+        <v>100</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B54" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C54" s="32" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D54" s="32" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E54" s="33" t="n">
         <v>6</v>
@@ -8347,19 +8936,23 @@
         <v>6</v>
       </c>
       <c r="P54" s="32"/>
+      <c r="Q54" s="35" t="n">
+        <f aca="false">E54*INDEX(요약!$C$4:$C$7,MATCH($A54,요약!$A$4:$A$7,0))</f>
+        <v>600</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B55" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C55" s="32" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D55" s="32" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E55" s="33" t="n">
         <v>4</v>
@@ -8405,19 +8998,23 @@
         <v>4</v>
       </c>
       <c r="P55" s="32"/>
+      <c r="Q55" s="35" t="n">
+        <f aca="false">E55*INDEX(요약!$C$4:$C$7,MATCH($A55,요약!$A$4:$A$7,0))</f>
+        <v>400</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B56" s="16" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C56" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D56" s="32" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E56" s="33" t="n">
         <v>1</v>
@@ -8463,71 +9060,76 @@
         <v>1</v>
       </c>
       <c r="P56" s="32"/>
+      <c r="Q56" s="35" t="n">
+        <f aca="false">E56*INDEX(요약!$C$4:$C$7,MATCH($A56,요약!$A$4:$A$7,0))</f>
+        <v>100</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="10" t="s">
+      <c r="A57" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B57" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="C57" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="D57" s="35" t="s">
+      <c r="B57" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="E57" s="35"/>
-      <c r="F57" s="35"/>
-      <c r="G57" s="11" t="n">
+      <c r="C57" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="D57" s="36" t="s">
+        <v>108</v>
+      </c>
+      <c r="E57" s="36"/>
+      <c r="F57" s="36"/>
+      <c r="G57" s="10" t="n">
         <f aca="false">SUM(G53:G56)</f>
         <v>1449500</v>
       </c>
-      <c r="H57" s="36" t="n">
+      <c r="H57" s="37" t="n">
         <f aca="false">SUM(H53:H56)</f>
         <v>110</v>
       </c>
-      <c r="I57" s="36" t="n">
+      <c r="I57" s="37" t="n">
         <f aca="false">SUM(I53:I56)</f>
         <v>10</v>
       </c>
-      <c r="J57" s="36" t="n">
+      <c r="J57" s="37" t="n">
         <f aca="false">SUM(J53:J56)</f>
         <v>64</v>
       </c>
-      <c r="K57" s="36" t="n">
+      <c r="K57" s="37" t="n">
         <f aca="false">SUM(K53:K56)</f>
         <v>74</v>
       </c>
-      <c r="L57" s="36" t="n">
+      <c r="L57" s="37" t="n">
         <f aca="false">SUM(L53:L56)</f>
         <v>4</v>
       </c>
-      <c r="M57" s="36" t="n">
+      <c r="M57" s="37" t="n">
         <f aca="false">SUM(M53:M56)</f>
         <v>2</v>
       </c>
-      <c r="N57" s="36" t="n">
+      <c r="N57" s="37" t="n">
         <f aca="false">SUM(N53:N56)</f>
         <v>1</v>
       </c>
-      <c r="O57" s="36" t="n">
+      <c r="O57" s="37" t="n">
         <f aca="false">SUM(O53:O56)</f>
         <v>11</v>
       </c>
-      <c r="P57" s="10" t="str">
+      <c r="P57" s="9" t="str">
         <f aca="false">IF(AND(H57&gt;=H42,K57&gt;=K42,J57&gt;=K42,L57&gt;=L42,M57&gt;=M42,N57&gt;=N42),IF(O57&gt;7,"OK (TM3 버스확장 필요)","OK"),"사양 미달")</f>
         <v>OK (TM3 버스확장 필요)</v>
       </c>
+      <c r="Q57" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="A5:P5"/>
-    <mergeCell ref="A15:P15"/>
-    <mergeCell ref="A28:P28"/>
-    <mergeCell ref="A41:P41"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A5:Q5"/>
+    <mergeCell ref="A15:Q15"/>
+    <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="A41:Q41"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -8538,4 +9140,855 @@
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I24"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="38" t="s">
+        <v>129</v>
+      </c>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="39" t="str">
+        <f aca="false">'Price List'!C3</f>
+        <v>TM241CE24T</v>
+      </c>
+      <c r="B5" s="39" t="str">
+        <f aca="false">'Price List'!R3</f>
+        <v>CPU, Ethernet, 24VDC</v>
+      </c>
+      <c r="C5" s="40" t="n">
+        <f aca="false">'Price List'!I3</f>
+        <v>398700</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A5,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>100</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <f aca="false">D5*$C5</f>
+        <v>39870000</v>
+      </c>
+      <c r="F5" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A5,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>100</v>
+      </c>
+      <c r="G5" s="20" t="n">
+        <f aca="false">F5*$C5</f>
+        <v>39870000</v>
+      </c>
+      <c r="H5" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A5,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>100</v>
+      </c>
+      <c r="I5" s="20" t="n">
+        <f aca="false">H5*$C5</f>
+        <v>39870000</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="39" t="str">
+        <f aca="false">'Price List'!C4</f>
+        <v>TM241C24T</v>
+      </c>
+      <c r="B6" s="39" t="str">
+        <f aca="false">'Price List'!R4</f>
+        <v>CPU, 24VDC</v>
+      </c>
+      <c r="C6" s="40" t="n">
+        <f aca="false">'Price List'!I4</f>
+        <v>392850</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A6,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>550</v>
+      </c>
+      <c r="E6" s="20" t="n">
+        <f aca="false">D6*$C6</f>
+        <v>216067500</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A6,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>250</v>
+      </c>
+      <c r="G6" s="20" t="n">
+        <f aca="false">F6*$C6</f>
+        <v>98212500</v>
+      </c>
+      <c r="H6" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A6,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="20" t="n">
+        <f aca="false">H6*$C6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="39" t="str">
+        <f aca="false">'Price List'!C5</f>
+        <v>TM241C24R</v>
+      </c>
+      <c r="B7" s="39" t="str">
+        <f aca="false">'Price List'!R5</f>
+        <v>CPU, 100-240VAC</v>
+      </c>
+      <c r="C7" s="40" t="n">
+        <f aca="false">'Price List'!I5</f>
+        <v>384750</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A7,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <f aca="false">D7*$C7</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A7,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="20" t="n">
+        <f aca="false">F7*$C7</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A7,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>250</v>
+      </c>
+      <c r="I7" s="20" t="n">
+        <f aca="false">H7*$C7</f>
+        <v>96187500</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="39" t="str">
+        <f aca="false">'Price List'!C6</f>
+        <v>TM241C40T</v>
+      </c>
+      <c r="B8" s="39" t="str">
+        <f aca="false">'Price List'!R6</f>
+        <v>CPU, 24VDC</v>
+      </c>
+      <c r="C8" s="40" t="n">
+        <f aca="false">'Price List'!I6</f>
+        <v>417600</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A8,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <f aca="false">D8*$C8</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A8,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>300</v>
+      </c>
+      <c r="G8" s="20" t="n">
+        <f aca="false">F8*$C8</f>
+        <v>125280000</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A8,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="20" t="n">
+        <f aca="false">H8*$C8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="39" t="str">
+        <f aca="false">'Price List'!C7</f>
+        <v>TM241C40R</v>
+      </c>
+      <c r="B9" s="39" t="str">
+        <f aca="false">'Price List'!R7</f>
+        <v>CPU, 100-240VAC</v>
+      </c>
+      <c r="C9" s="40" t="n">
+        <f aca="false">'Price List'!I7</f>
+        <v>406350</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A9,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <f aca="false">D9*$C9</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A9,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="20" t="n">
+        <f aca="false">F9*$C9</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A9,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>300</v>
+      </c>
+      <c r="I9" s="20" t="n">
+        <f aca="false">H9*$C9</f>
+        <v>121905000</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="39" t="str">
+        <f aca="false">'Price List'!C8</f>
+        <v>TM3DI16</v>
+      </c>
+      <c r="B10" s="39" t="str">
+        <f aca="false">'Price List'!R8</f>
+        <v>DI 16</v>
+      </c>
+      <c r="C10" s="40" t="n">
+        <f aca="false">'Price List'!I8</f>
+        <v>91200</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A10,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>600</v>
+      </c>
+      <c r="E10" s="20" t="n">
+        <f aca="false">D10*$C10</f>
+        <v>54720000</v>
+      </c>
+      <c r="F10" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A10,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>600</v>
+      </c>
+      <c r="G10" s="20" t="n">
+        <f aca="false">F10*$C10</f>
+        <v>54720000</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A10,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>600</v>
+      </c>
+      <c r="I10" s="20" t="n">
+        <f aca="false">H10*$C10</f>
+        <v>54720000</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="39" t="str">
+        <f aca="false">'Price List'!C9</f>
+        <v>TM3DI8</v>
+      </c>
+      <c r="B11" s="39" t="str">
+        <f aca="false">'Price List'!R9</f>
+        <v>DI 8</v>
+      </c>
+      <c r="C11" s="40" t="n">
+        <f aca="false">'Price List'!I9</f>
+        <v>80800</v>
+      </c>
+      <c r="D11" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A11,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="20" t="n">
+        <f aca="false">D11*$C11</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A11,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="20" t="n">
+        <f aca="false">F11*$C11</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A11,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="20" t="n">
+        <f aca="false">H11*$C11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="39" t="str">
+        <f aca="false">'Price List'!C10</f>
+        <v>TM3DQ16R</v>
+      </c>
+      <c r="B12" s="39" t="str">
+        <f aca="false">'Price List'!R10</f>
+        <v>DO 16 Relay</v>
+      </c>
+      <c r="C12" s="40" t="n">
+        <f aca="false">'Price List'!I10</f>
+        <v>90800</v>
+      </c>
+      <c r="D12" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A12,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>700</v>
+      </c>
+      <c r="E12" s="20" t="n">
+        <f aca="false">D12*$C12</f>
+        <v>63560000</v>
+      </c>
+      <c r="F12" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A12,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="20" t="n">
+        <f aca="false">F12*$C12</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A12,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>400</v>
+      </c>
+      <c r="I12" s="20" t="n">
+        <f aca="false">H12*$C12</f>
+        <v>36320000</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="39" t="str">
+        <f aca="false">'Price List'!C11</f>
+        <v>TM3DQ16T</v>
+      </c>
+      <c r="B13" s="39" t="str">
+        <f aca="false">'Price List'!R11</f>
+        <v>DO 16 Tr (Source)</v>
+      </c>
+      <c r="C13" s="40" t="n">
+        <f aca="false">'Price List'!I11</f>
+        <v>90800</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A13,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="20" t="n">
+        <f aca="false">D13*$C13</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A13,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>300</v>
+      </c>
+      <c r="G13" s="20" t="n">
+        <f aca="false">F13*$C13</f>
+        <v>27240000</v>
+      </c>
+      <c r="H13" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A13,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="20" t="n">
+        <f aca="false">H13*$C13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="39" t="str">
+        <f aca="false">'Price List'!C12</f>
+        <v>TM3DQ16U</v>
+      </c>
+      <c r="B14" s="39" t="str">
+        <f aca="false">'Price List'!R12</f>
+        <v>DO 16 Tr (Sink)</v>
+      </c>
+      <c r="C14" s="40" t="n">
+        <f aca="false">'Price List'!I12</f>
+        <v>85200</v>
+      </c>
+      <c r="D14" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A14,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="20" t="n">
+        <f aca="false">D14*$C14</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A14,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="20" t="n">
+        <f aca="false">F14*$C14</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A14,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="20" t="n">
+        <f aca="false">H14*$C14</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="39" t="str">
+        <f aca="false">'Price List'!C13</f>
+        <v>TM3DQ8R</v>
+      </c>
+      <c r="B15" s="39" t="str">
+        <f aca="false">'Price List'!R13</f>
+        <v>DO 8 Relay</v>
+      </c>
+      <c r="C15" s="40" t="n">
+        <f aca="false">'Price List'!I13</f>
+        <v>64400</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A15,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>250</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <f aca="false">D15*$C15</f>
+        <v>16100000</v>
+      </c>
+      <c r="F15" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A15,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="20" t="n">
+        <f aca="false">F15*$C15</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A15,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="20" t="n">
+        <f aca="false">H15*$C15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="39" t="str">
+        <f aca="false">'Price List'!C14</f>
+        <v>TM3DQ8T</v>
+      </c>
+      <c r="B16" s="39" t="str">
+        <f aca="false">'Price List'!R14</f>
+        <v>DO 8 Tr (Source)</v>
+      </c>
+      <c r="C16" s="40" t="n">
+        <f aca="false">'Price List'!I14</f>
+        <v>67200</v>
+      </c>
+      <c r="D16" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A16,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="20" t="n">
+        <f aca="false">D16*$C16</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A16,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="20" t="n">
+        <f aca="false">F16*$C16</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A16,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="20" t="n">
+        <f aca="false">H16*$C16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="39" t="str">
+        <f aca="false">'Price List'!C15</f>
+        <v>TM3DQ8U</v>
+      </c>
+      <c r="B17" s="39" t="str">
+        <f aca="false">'Price List'!R15</f>
+        <v>DO 8 Tr (Sink)</v>
+      </c>
+      <c r="C17" s="40" t="n">
+        <f aca="false">'Price List'!I15</f>
+        <v>67200</v>
+      </c>
+      <c r="D17" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A17,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="20" t="n">
+        <f aca="false">D17*$C17</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A17,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="20" t="n">
+        <f aca="false">F17*$C17</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A17,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="20" t="n">
+        <f aca="false">H17*$C17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="39" t="str">
+        <f aca="false">'Price List'!C16</f>
+        <v>TM3AI2H</v>
+      </c>
+      <c r="B18" s="39" t="str">
+        <f aca="false">'Price List'!R16</f>
+        <v>AI 2 (16bit)</v>
+      </c>
+      <c r="C18" s="40" t="n">
+        <f aca="false">'Price List'!I16</f>
+        <v>124400</v>
+      </c>
+      <c r="D18" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A18,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="20" t="n">
+        <f aca="false">D18*$C18</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A18,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="20" t="n">
+        <f aca="false">F18*$C18</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A18,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="20" t="n">
+        <f aca="false">H18*$C18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="39" t="str">
+        <f aca="false">'Price List'!C17</f>
+        <v>TM3AI4</v>
+      </c>
+      <c r="B19" s="39" t="str">
+        <f aca="false">'Price List'!R17</f>
+        <v>AI 4</v>
+      </c>
+      <c r="C19" s="40" t="n">
+        <f aca="false">'Price List'!I17</f>
+        <v>113600</v>
+      </c>
+      <c r="D19" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A19,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="20" t="n">
+        <f aca="false">D19*$C19</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A19,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="20" t="n">
+        <f aca="false">F19*$C19</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A19,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I19" s="20" t="n">
+        <f aca="false">H19*$C19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="39" t="str">
+        <f aca="false">'Price List'!C18</f>
+        <v>TM3AI8</v>
+      </c>
+      <c r="B20" s="39" t="str">
+        <f aca="false">'Price List'!R18</f>
+        <v>AI 8</v>
+      </c>
+      <c r="C20" s="40" t="n">
+        <f aca="false">'Price List'!I18</f>
+        <v>132400</v>
+      </c>
+      <c r="D20" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A20,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="20" t="n">
+        <f aca="false">D20*$C20</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A20,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="20" t="n">
+        <f aca="false">F20*$C20</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A20,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="20" t="n">
+        <f aca="false">H20*$C20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="39" t="str">
+        <f aca="false">'Price List'!C19</f>
+        <v>TM3AQ2</v>
+      </c>
+      <c r="B21" s="39" t="str">
+        <f aca="false">'Price List'!R19</f>
+        <v>AO 2</v>
+      </c>
+      <c r="C21" s="40" t="n">
+        <f aca="false">'Price List'!I19</f>
+        <v>138400</v>
+      </c>
+      <c r="D21" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A21,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>350</v>
+      </c>
+      <c r="E21" s="20" t="n">
+        <f aca="false">D21*$C21</f>
+        <v>48440000</v>
+      </c>
+      <c r="F21" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A21,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>350</v>
+      </c>
+      <c r="G21" s="20" t="n">
+        <f aca="false">F21*$C21</f>
+        <v>48440000</v>
+      </c>
+      <c r="H21" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A21,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>350</v>
+      </c>
+      <c r="I21" s="20" t="n">
+        <f aca="false">H21*$C21</f>
+        <v>48440000</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="39" t="str">
+        <f aca="false">'Price List'!C20</f>
+        <v>TM3AQ4</v>
+      </c>
+      <c r="B22" s="39" t="str">
+        <f aca="false">'Price List'!R20</f>
+        <v>AO 4</v>
+      </c>
+      <c r="C22" s="40" t="n">
+        <f aca="false">'Price List'!I20</f>
+        <v>140400</v>
+      </c>
+      <c r="D22" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A22,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>100</v>
+      </c>
+      <c r="E22" s="20" t="n">
+        <f aca="false">D22*$C22</f>
+        <v>14040000</v>
+      </c>
+      <c r="F22" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A22,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>100</v>
+      </c>
+      <c r="G22" s="20" t="n">
+        <f aca="false">F22*$C22</f>
+        <v>14040000</v>
+      </c>
+      <c r="H22" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A22,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>100</v>
+      </c>
+      <c r="I22" s="20" t="n">
+        <f aca="false">H22*$C22</f>
+        <v>14040000</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="36"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="10" t="n">
+        <f aca="false">SUM(D5:D22)</f>
+        <v>2650</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <f aca="false">SUM(E5:E22)</f>
+        <v>452797500</v>
+      </c>
+      <c r="F23" s="10" t="n">
+        <f aca="false">SUM(F5:F22)</f>
+        <v>2000</v>
+      </c>
+      <c r="G23" s="10" t="n">
+        <f aca="false">SUM(G5:G22)</f>
+        <v>407802500</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <f aca="false">SUM(H5:H22)</f>
+        <v>2100</v>
+      </c>
+      <c r="I23" s="10" t="n">
+        <f aca="false">SUM(I5:I22)</f>
+        <v>411482500</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="B24" s="41"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="42"/>
+      <c r="E24" s="42" t="str">
+        <f aca="false">IF(ABS(E23-요약!G8)&lt;1,"일치","불일치")</f>
+        <v>일치</v>
+      </c>
+      <c r="F24" s="42"/>
+      <c r="G24" s="42" t="str">
+        <f aca="false">IF(ABS(G23-요약!H8)&lt;1,"일치","불일치")</f>
+        <v>일치</v>
+      </c>
+      <c r="H24" s="42"/>
+      <c r="I24" s="42" t="str">
+        <f aca="false">IF(ABS(I23-요약!I8)&lt;1,"일치","불일치")</f>
+        <v>일치</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A24:C24"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add CPU discount factor comparison sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjFrCobQqqs1TtLcuKd8BA
</commit_message>
<xml_diff>
--- a/IDMST_Price_List.xlsx
+++ b/IDMST_Price_List.xlsx
@@ -13,6 +13,7 @@
     <sheet name="기준사양 매칭" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="연간 BOM" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Schneider 제안 검토" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="CPU DF 비교" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -653,8 +654,110 @@
 </comments>
 </file>
 
+<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Schneider MCC </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">제안 </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">CPU — </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">가격표에 없어 추정 정가</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">(Schneider </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">제안 검토</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">!B5) </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">사용</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">. </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">제 안에는 쓰이지 않아 수량 </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">0.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="183">
   <si>
     <r>
       <rPr>
@@ -6785,6 +6888,627 @@
       <rPr>
         <sz val="10"/>
         <color rgb="FF262626"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CPU </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">할인율</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(DF) </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">변경 시 매입가 차이</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">현재 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DF</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">협상 목표 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DF</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">← 이 칸을 바꾸면 전체 재계산</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List Price</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">현재 단가
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">현재 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DF)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목표 단가
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목표 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DF)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단가 차이
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1EA)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 수량
+안</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">B (DC24V)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 절감
+안</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">B</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 수량
+안</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">C (AC220V)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 절감
+안</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">C</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 단가 차이 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= List Price × (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">현재 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DF − </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목표 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DF). 0.45 → 0.40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이면 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">List Price</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5%.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 연간 수량은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">BOM' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연간 구매수량 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">구성안별 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CPU </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수량</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에서 가져옴</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. TM3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확장 모듈 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DF(0.40)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 그대로 두었음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">• TM241CE40T</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Schneider MCC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제안용 추정 정가 기준 참고값</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF404040"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
@@ -6804,7 +7528,7 @@
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0;\-0;\-"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="36">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -7023,6 +7747,30 @@
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -7105,7 +7853,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="71">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -7340,6 +8088,54 @@
     </xf>
     <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="33" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -14548,4 +15344,423 @@
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="43" t="s">
+        <v>167</v>
+      </c>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="59" t="s">
+        <v>168</v>
+      </c>
+      <c r="B3" s="60" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="59" t="s">
+        <v>169</v>
+      </c>
+      <c r="B4" s="60" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C4" s="61" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="62" t="str">
+        <f aca="false">'Price List'!C3</f>
+        <v>TM241CE24T</v>
+      </c>
+      <c r="B7" s="63" t="str">
+        <f aca="false">'Price List'!D3</f>
+        <v>DC</v>
+      </c>
+      <c r="C7" s="40" t="n">
+        <f aca="false">'Price List'!F3</f>
+        <v>886000</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <f aca="false">ROUND(C7*$B$3,0)</f>
+        <v>398700</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <f aca="false">ROUND(C7*$B$4,0)</f>
+        <v>354400</v>
+      </c>
+      <c r="F7" s="64" t="n">
+        <f aca="false">D7-E7</f>
+        <v>44300</v>
+      </c>
+      <c r="G7" s="40" t="n">
+        <f aca="false">INDEX('연간 BOM'!$F$5:$F$22,MATCH($A7,'연간 BOM'!$A$5:$A$22,0))</f>
+        <v>100</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <f aca="false">F7*G7</f>
+        <v>4430000</v>
+      </c>
+      <c r="I7" s="40" t="n">
+        <f aca="false">INDEX('연간 BOM'!$H$5:$H$22,MATCH($A7,'연간 BOM'!$A$5:$A$22,0))</f>
+        <v>100</v>
+      </c>
+      <c r="J7" s="20" t="n">
+        <f aca="false">F7*I7</f>
+        <v>4430000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="62" t="str">
+        <f aca="false">'Price List'!C4</f>
+        <v>TM241C24T</v>
+      </c>
+      <c r="B8" s="63" t="str">
+        <f aca="false">'Price List'!D4</f>
+        <v>DC</v>
+      </c>
+      <c r="C8" s="40" t="n">
+        <f aca="false">'Price List'!F4</f>
+        <v>873000</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <f aca="false">ROUND(C8*$B$3,0)</f>
+        <v>392850</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <f aca="false">ROUND(C8*$B$4,0)</f>
+        <v>349200</v>
+      </c>
+      <c r="F8" s="64" t="n">
+        <f aca="false">D8-E8</f>
+        <v>43650</v>
+      </c>
+      <c r="G8" s="40" t="n">
+        <f aca="false">INDEX('연간 BOM'!$F$5:$F$22,MATCH($A8,'연간 BOM'!$A$5:$A$22,0))</f>
+        <v>250</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <f aca="false">F8*G8</f>
+        <v>10912500</v>
+      </c>
+      <c r="I8" s="40" t="n">
+        <f aca="false">INDEX('연간 BOM'!$H$5:$H$22,MATCH($A8,'연간 BOM'!$A$5:$A$22,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="20" t="n">
+        <f aca="false">F8*I8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="62" t="str">
+        <f aca="false">'Price List'!C5</f>
+        <v>TM241C24R</v>
+      </c>
+      <c r="B9" s="63" t="str">
+        <f aca="false">'Price List'!D5</f>
+        <v>AC</v>
+      </c>
+      <c r="C9" s="40" t="n">
+        <f aca="false">'Price List'!F5</f>
+        <v>855000</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <f aca="false">ROUND(C9*$B$3,0)</f>
+        <v>384750</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <f aca="false">ROUND(C9*$B$4,0)</f>
+        <v>342000</v>
+      </c>
+      <c r="F9" s="64" t="n">
+        <f aca="false">D9-E9</f>
+        <v>42750</v>
+      </c>
+      <c r="G9" s="40" t="n">
+        <f aca="false">INDEX('연간 BOM'!$F$5:$F$22,MATCH($A9,'연간 BOM'!$A$5:$A$22,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <f aca="false">F9*G9</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="40" t="n">
+        <f aca="false">INDEX('연간 BOM'!$H$5:$H$22,MATCH($A9,'연간 BOM'!$A$5:$A$22,0))</f>
+        <v>250</v>
+      </c>
+      <c r="J9" s="20" t="n">
+        <f aca="false">F9*I9</f>
+        <v>10687500</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="62" t="str">
+        <f aca="false">'Price List'!C6</f>
+        <v>TM241C40T</v>
+      </c>
+      <c r="B10" s="63" t="str">
+        <f aca="false">'Price List'!D6</f>
+        <v>DC</v>
+      </c>
+      <c r="C10" s="40" t="n">
+        <f aca="false">'Price List'!F6</f>
+        <v>928000</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <f aca="false">ROUND(C10*$B$3,0)</f>
+        <v>417600</v>
+      </c>
+      <c r="E10" s="20" t="n">
+        <f aca="false">ROUND(C10*$B$4,0)</f>
+        <v>371200</v>
+      </c>
+      <c r="F10" s="64" t="n">
+        <f aca="false">D10-E10</f>
+        <v>46400</v>
+      </c>
+      <c r="G10" s="40" t="n">
+        <f aca="false">INDEX('연간 BOM'!$F$5:$F$22,MATCH($A10,'연간 BOM'!$A$5:$A$22,0))</f>
+        <v>300</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <f aca="false">F10*G10</f>
+        <v>13920000</v>
+      </c>
+      <c r="I10" s="40" t="n">
+        <f aca="false">INDEX('연간 BOM'!$H$5:$H$22,MATCH($A10,'연간 BOM'!$A$5:$A$22,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="20" t="n">
+        <f aca="false">F10*I10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="62" t="str">
+        <f aca="false">'Price List'!C7</f>
+        <v>TM241C40R</v>
+      </c>
+      <c r="B11" s="63" t="str">
+        <f aca="false">'Price List'!D7</f>
+        <v>AC</v>
+      </c>
+      <c r="C11" s="40" t="n">
+        <f aca="false">'Price List'!F7</f>
+        <v>903000</v>
+      </c>
+      <c r="D11" s="20" t="n">
+        <f aca="false">ROUND(C11*$B$3,0)</f>
+        <v>406350</v>
+      </c>
+      <c r="E11" s="20" t="n">
+        <f aca="false">ROUND(C11*$B$4,0)</f>
+        <v>361200</v>
+      </c>
+      <c r="F11" s="64" t="n">
+        <f aca="false">D11-E11</f>
+        <v>45150</v>
+      </c>
+      <c r="G11" s="40" t="n">
+        <f aca="false">INDEX('연간 BOM'!$F$5:$F$22,MATCH($A11,'연간 BOM'!$A$5:$A$22,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="20" t="n">
+        <f aca="false">F11*G11</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="40" t="n">
+        <f aca="false">INDEX('연간 BOM'!$H$5:$H$22,MATCH($A11,'연간 BOM'!$A$5:$A$22,0))</f>
+        <v>300</v>
+      </c>
+      <c r="J11" s="20" t="n">
+        <f aca="false">F11*I11</f>
+        <v>13545000</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="65" t="str">
+        <f aca="false">'Schneider 제안 검토'!A5</f>
+        <v>TM241CE40T</v>
+      </c>
+      <c r="B12" s="66" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="67" t="n">
+        <f aca="false">'Schneider 제안 검토'!B5</f>
+        <v>941000</v>
+      </c>
+      <c r="D12" s="68" t="n">
+        <f aca="false">ROUND(C12*$B$3,0)</f>
+        <v>423450</v>
+      </c>
+      <c r="E12" s="68" t="n">
+        <f aca="false">ROUND(C12*$B$4,0)</f>
+        <v>376400</v>
+      </c>
+      <c r="F12" s="64" t="n">
+        <f aca="false">D12-E12</f>
+        <v>47050</v>
+      </c>
+      <c r="G12" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="68" t="n">
+        <f aca="false">F12*G12</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="68" t="n">
+        <f aca="false">F12*I12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="36"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="10" t="n">
+        <f aca="false">SUM(G7:G12)</f>
+        <v>650</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <f aca="false">SUM(H7:H12)</f>
+        <v>29262500</v>
+      </c>
+      <c r="I13" s="10" t="n">
+        <f aca="false">SUM(I7:I12)</f>
+        <v>650</v>
+      </c>
+      <c r="J13" s="10" t="n">
+        <f aca="false">SUM(J7:J12)</f>
+        <v>28662500</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="69" t="s">
+        <v>180</v>
+      </c>
+      <c r="B15" s="69"/>
+      <c r="C15" s="69"/>
+      <c r="D15" s="69"/>
+      <c r="E15" s="69"/>
+      <c r="F15" s="69"/>
+      <c r="G15" s="69"/>
+      <c r="H15" s="69"/>
+      <c r="I15" s="69"/>
+      <c r="J15" s="69"/>
+    </row>
+    <row r="16" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="69" t="s">
+        <v>181</v>
+      </c>
+      <c r="B16" s="69"/>
+      <c r="C16" s="69"/>
+      <c r="D16" s="69"/>
+      <c r="E16" s="69"/>
+      <c r="F16" s="69"/>
+      <c r="G16" s="69"/>
+      <c r="H16" s="69"/>
+      <c r="I16" s="69"/>
+      <c r="J16" s="69"/>
+    </row>
+    <row r="17" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="70" t="s">
+        <v>182</v>
+      </c>
+      <c r="B17" s="70"/>
+      <c r="C17" s="70"/>
+      <c r="D17" s="70"/>
+      <c r="E17" s="70"/>
+      <c r="F17" s="70"/>
+      <c r="G17" s="70"/>
+      <c r="H17" s="70"/>
+      <c r="I17" s="70"/>
+      <c r="J17" s="70"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A15:J15"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A17:J17"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add TM241CE40T and TM3 bus expansion prices to original price list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjFrCobQqqs1TtLcuKd8BA
</commit_message>
<xml_diff>
--- a/IDMST_Price_List.xlsx
+++ b/IDMST_Price_List.xlsx
@@ -30,7 +30,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="H21" authorId="0">
+    <comment ref="H24" authorId="0">
       <text>
         <r>
           <rPr>
@@ -757,7 +757,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="188">
   <si>
     <r>
       <rPr>
@@ -2416,6 +2416,146 @@
     <t xml:space="preserve">AO 4</t>
   </si>
   <si>
+    <t xml:space="preserve">TM241CE40T</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CPU, Ethernet, 24VDC (10/06 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">추가 견적</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">TM3XTRA1</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TM3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">버스 확장 송신 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(10/06 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">추가 견적</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">TM3XREC1</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TM3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">버스 확장 수신 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(10/06 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">추가 견적</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">Total</t>
   </si>
   <si>
@@ -2722,7 +2862,70 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">.</t>
+      <t xml:space="preserve">. 19~21</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">번은 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026-10-06 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">추가 견적 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">참고 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NP: 579,600 / 98,280 / 116,550).</t>
     </r>
   </si>
   <si>
@@ -4972,9 +5175,6 @@
   </si>
   <si>
     <t xml:space="preserve">근거</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TM241CE40T</t>
   </si>
   <si>
     <r>
@@ -7640,6 +7840,12 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
       <i val="true"/>
       <sz val="9"/>
       <color rgb="FF595959"/>
@@ -7676,12 +7882,6 @@
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FF1F3864"/>
-      <name val="WenQuanYi Zen Hei"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
     </font>
@@ -7958,15 +8158,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8006,7 +8206,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8062,7 +8262,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8078,7 +8278,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8098,7 +8298,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8770,7 +8970,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -9908,52 +10108,225 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="9" t="n">
-        <f aca="false">SUM(E3:E20)</f>
-        <v>18</v>
-      </c>
-      <c r="F21" s="24"/>
-      <c r="G21" s="10" t="n">
-        <f aca="false">SUM(G3:G20)</f>
-        <v>7662000</v>
-      </c>
-      <c r="H21" s="25" t="n">
-        <f aca="false">IFERROR(J21/G21,0)</f>
-        <v>0.429006786739755</v>
-      </c>
-      <c r="I21" s="24"/>
-      <c r="J21" s="10" t="n">
-        <f aca="false">SUM(J3:J20)</f>
-        <v>3287050</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="26" t="s">
+      <c r="D21" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <v>920000</v>
+      </c>
+      <c r="G21" s="20" t="n">
+        <f aca="false">E21*F21</f>
+        <v>920000</v>
+      </c>
+      <c r="H21" s="21" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I21" s="20" t="n">
+        <f aca="false">ROUND(F21*H21,0)</f>
+        <v>414000</v>
+      </c>
+      <c r="J21" s="20" t="n">
+        <f aca="false">E21*I21</f>
+        <v>414000</v>
+      </c>
+      <c r="K21" s="22" t="n">
+        <v>24</v>
+      </c>
+      <c r="L21" s="22" t="n">
+        <v>16</v>
+      </c>
+      <c r="M21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q21" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="R21" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26"/>
-      <c r="I23" s="26"/>
-      <c r="J23" s="26"/>
-      <c r="K23" s="26"/>
-      <c r="L23" s="26"/>
-      <c r="M23" s="26"/>
-      <c r="N23" s="26"/>
-      <c r="O23" s="26"/>
-      <c r="P23" s="26"/>
-      <c r="Q23" s="26"/>
-      <c r="R23" s="26"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="D22" s="16"/>
+      <c r="E22" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="19" t="n">
+        <v>156000</v>
+      </c>
+      <c r="G22" s="20" t="n">
+        <f aca="false">E22*F22</f>
+        <v>156000</v>
+      </c>
+      <c r="H22" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I22" s="20" t="n">
+        <f aca="false">ROUND(F22*H22,0)</f>
+        <v>62400</v>
+      </c>
+      <c r="J22" s="20" t="n">
+        <f aca="false">E22*I22</f>
+        <v>62400</v>
+      </c>
+      <c r="K22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="17" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="D23" s="16"/>
+      <c r="E23" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="19" t="n">
+        <v>185000</v>
+      </c>
+      <c r="G23" s="20" t="n">
+        <f aca="false">E23*F23</f>
+        <v>185000</v>
+      </c>
+      <c r="H23" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I23" s="20" t="n">
+        <f aca="false">ROUND(F23*H23,0)</f>
+        <v>74000</v>
+      </c>
+      <c r="J23" s="20" t="n">
+        <f aca="false">E23*I23</f>
+        <v>74000</v>
+      </c>
+      <c r="K23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="17" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="23"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="9" t="n">
+        <f aca="false">SUM(E3:E23)</f>
+        <v>21</v>
+      </c>
+      <c r="F24" s="24"/>
+      <c r="G24" s="10" t="n">
+        <f aca="false">SUM(G3:G23)</f>
+        <v>8923000</v>
+      </c>
+      <c r="H24" s="25" t="n">
+        <f aca="false">IFERROR(J24/G24,0)</f>
+        <v>0.430062759161717</v>
+      </c>
+      <c r="I24" s="24"/>
+      <c r="J24" s="10" t="n">
+        <f aca="false">SUM(J3:J23)</f>
+        <v>3837450</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="B26" s="26"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="26"/>
+      <c r="I26" s="26"/>
+      <c r="J26" s="26"/>
+      <c r="K26" s="26"/>
+      <c r="L26" s="26"/>
+      <c r="M26" s="26"/>
+      <c r="N26" s="26"/>
+      <c r="O26" s="26"/>
+      <c r="P26" s="26"/>
+      <c r="Q26" s="26"/>
+      <c r="R26" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -9965,8 +10338,8 @@
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="K1:R1"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A23:R23"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A26:R26"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -10008,7 +10381,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -10029,7 +10402,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="27" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -10053,22 +10426,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C4" s="15" t="s">
         <v>30</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>32</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="H4" s="15" t="s">
         <v>39</v>
@@ -10080,7 +10453,7 @@
         <v>41</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="L4" s="15" t="s">
         <v>43</v>
@@ -10092,18 +10465,18 @@
         <v>45</v>
       </c>
       <c r="O4" s="15" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B5" s="28"/>
       <c r="C5" s="28"/>
@@ -10127,11 +10500,11 @@
         <v>10</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C6" s="30"/>
       <c r="D6" s="31" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="E6" s="30"/>
       <c r="F6" s="30"/>
@@ -10162,19 +10535,19 @@
         <v>10</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C7" s="32" t="s">
         <v>51</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E7" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C7,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C7,'Price List'!$C$3:$C$23,0))</f>
         <v>392850</v>
       </c>
       <c r="G7" s="20" t="n">
@@ -10182,15 +10555,15 @@
         <v>392850</v>
       </c>
       <c r="H7" s="34" t="n">
-        <f aca="false">E7*INDEX('Price List'!$K$3:$K$20,MATCH($C7,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E7*INDEX('Price List'!$K$3:$K$23,MATCH($C7,'Price List'!$C$3:$C$23,0))</f>
         <v>14</v>
       </c>
       <c r="I7" s="34" t="n">
-        <f aca="false">E7*INDEX('Price List'!$L$3:$L$20,MATCH($C7,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E7*INDEX('Price List'!$L$3:$L$23,MATCH($C7,'Price List'!$C$3:$C$23,0))</f>
         <v>10</v>
       </c>
       <c r="J7" s="34" t="n">
-        <f aca="false">E7*INDEX('Price List'!$M$3:$M$20,MATCH($C7,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E7*INDEX('Price List'!$M$3:$M$23,MATCH($C7,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K7" s="34" t="n">
@@ -10198,15 +10571,15 @@
         <v>10</v>
       </c>
       <c r="L7" s="34" t="n">
-        <f aca="false">E7*INDEX('Price List'!$O$3:$O$20,MATCH($C7,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E7*INDEX('Price List'!$O$3:$O$23,MATCH($C7,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M7" s="34" t="n">
-        <f aca="false">E7*INDEX('Price List'!$P$3:$P$20,MATCH($C7,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E7*INDEX('Price List'!$P$3:$P$23,MATCH($C7,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="N7" s="34" t="n">
-        <f aca="false">E7*INDEX('Price List'!$Q$3:$Q$20,MATCH($C7,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E7*INDEX('Price List'!$Q$3:$Q$23,MATCH($C7,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O7" s="34" t="n">
@@ -10224,19 +10597,19 @@
         <v>10</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C8" s="32" t="s">
         <v>68</v>
       </c>
       <c r="D8" s="32" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="E8" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C8,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C8,'Price List'!$C$3:$C$23,0))</f>
         <v>64400</v>
       </c>
       <c r="G8" s="20" t="n">
@@ -10244,15 +10617,15 @@
         <v>64400</v>
       </c>
       <c r="H8" s="34" t="n">
-        <f aca="false">E8*INDEX('Price List'!$K$3:$K$20,MATCH($C8,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E8*INDEX('Price List'!$K$3:$K$23,MATCH($C8,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I8" s="34" t="n">
-        <f aca="false">E8*INDEX('Price List'!$L$3:$L$20,MATCH($C8,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E8*INDEX('Price List'!$L$3:$L$23,MATCH($C8,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J8" s="34" t="n">
-        <f aca="false">E8*INDEX('Price List'!$M$3:$M$20,MATCH($C8,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E8*INDEX('Price List'!$M$3:$M$23,MATCH($C8,'Price List'!$C$3:$C$23,0))</f>
         <v>8</v>
       </c>
       <c r="K8" s="34" t="n">
@@ -10260,15 +10633,15 @@
         <v>8</v>
       </c>
       <c r="L8" s="34" t="n">
-        <f aca="false">E8*INDEX('Price List'!$O$3:$O$20,MATCH($C8,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E8*INDEX('Price List'!$O$3:$O$23,MATCH($C8,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M8" s="34" t="n">
-        <f aca="false">E8*INDEX('Price List'!$P$3:$P$20,MATCH($C8,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E8*INDEX('Price List'!$P$3:$P$23,MATCH($C8,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N8" s="34" t="n">
-        <f aca="false">E8*INDEX('Price List'!$Q$3:$Q$20,MATCH($C8,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E8*INDEX('Price List'!$Q$3:$Q$23,MATCH($C8,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O8" s="34" t="n">
@@ -10286,13 +10659,13 @@
         <v>10</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C9" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D9" s="36" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E9" s="36"/>
       <c r="F9" s="36"/>
@@ -10343,19 +10716,19 @@
         <v>10</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C10" s="32" t="s">
         <v>51</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E10" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C10,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C10,'Price List'!$C$3:$C$23,0))</f>
         <v>392850</v>
       </c>
       <c r="G10" s="20" t="n">
@@ -10363,15 +10736,15 @@
         <v>392850</v>
       </c>
       <c r="H10" s="34" t="n">
-        <f aca="false">E10*INDEX('Price List'!$K$3:$K$20,MATCH($C10,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E10*INDEX('Price List'!$K$3:$K$23,MATCH($C10,'Price List'!$C$3:$C$23,0))</f>
         <v>14</v>
       </c>
       <c r="I10" s="34" t="n">
-        <f aca="false">E10*INDEX('Price List'!$L$3:$L$20,MATCH($C10,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E10*INDEX('Price List'!$L$3:$L$23,MATCH($C10,'Price List'!$C$3:$C$23,0))</f>
         <v>10</v>
       </c>
       <c r="J10" s="34" t="n">
-        <f aca="false">E10*INDEX('Price List'!$M$3:$M$20,MATCH($C10,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E10*INDEX('Price List'!$M$3:$M$23,MATCH($C10,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K10" s="34" t="n">
@@ -10379,15 +10752,15 @@
         <v>10</v>
       </c>
       <c r="L10" s="34" t="n">
-        <f aca="false">E10*INDEX('Price List'!$O$3:$O$20,MATCH($C10,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E10*INDEX('Price List'!$O$3:$O$23,MATCH($C10,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M10" s="34" t="n">
-        <f aca="false">E10*INDEX('Price List'!$P$3:$P$20,MATCH($C10,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E10*INDEX('Price List'!$P$3:$P$23,MATCH($C10,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="N10" s="34" t="n">
-        <f aca="false">E10*INDEX('Price List'!$Q$3:$Q$20,MATCH($C10,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E10*INDEX('Price List'!$Q$3:$Q$23,MATCH($C10,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O10" s="34" t="n">
@@ -10405,13 +10778,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C11" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D11" s="36" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="E11" s="36"/>
       <c r="F11" s="36"/>
@@ -10462,19 +10835,19 @@
         <v>10</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C12" s="32" t="s">
         <v>53</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="E12" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C12,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C12,'Price List'!$C$3:$C$23,0))</f>
         <v>384750</v>
       </c>
       <c r="G12" s="20" t="n">
@@ -10482,15 +10855,15 @@
         <v>384750</v>
       </c>
       <c r="H12" s="34" t="n">
-        <f aca="false">E12*INDEX('Price List'!$K$3:$K$20,MATCH($C12,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E12*INDEX('Price List'!$K$3:$K$23,MATCH($C12,'Price List'!$C$3:$C$23,0))</f>
         <v>14</v>
       </c>
       <c r="I12" s="34" t="n">
-        <f aca="false">E12*INDEX('Price List'!$L$3:$L$20,MATCH($C12,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E12*INDEX('Price List'!$L$3:$L$23,MATCH($C12,'Price List'!$C$3:$C$23,0))</f>
         <v>4</v>
       </c>
       <c r="J12" s="34" t="n">
-        <f aca="false">E12*INDEX('Price List'!$M$3:$M$20,MATCH($C12,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E12*INDEX('Price List'!$M$3:$M$23,MATCH($C12,'Price List'!$C$3:$C$23,0))</f>
         <v>6</v>
       </c>
       <c r="K12" s="34" t="n">
@@ -10498,15 +10871,15 @@
         <v>10</v>
       </c>
       <c r="L12" s="34" t="n">
-        <f aca="false">E12*INDEX('Price List'!$O$3:$O$20,MATCH($C12,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E12*INDEX('Price List'!$O$3:$O$23,MATCH($C12,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M12" s="34" t="n">
-        <f aca="false">E12*INDEX('Price List'!$P$3:$P$20,MATCH($C12,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E12*INDEX('Price List'!$P$3:$P$23,MATCH($C12,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="N12" s="34" t="n">
-        <f aca="false">E12*INDEX('Price List'!$Q$3:$Q$20,MATCH($C12,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E12*INDEX('Price List'!$Q$3:$Q$23,MATCH($C12,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O12" s="34" t="n">
@@ -10524,13 +10897,13 @@
         <v>10</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C13" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D13" s="36" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E13" s="36"/>
       <c r="F13" s="36"/>
@@ -10578,7 +10951,7 @@
     </row>
     <row r="15" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B15" s="28"/>
       <c r="C15" s="28"/>
@@ -10602,11 +10975,11 @@
         <v>12</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C16" s="30"/>
       <c r="D16" s="31" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="E16" s="30"/>
       <c r="F16" s="30"/>
@@ -10637,19 +11010,19 @@
         <v>12</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C17" s="32" t="s">
         <v>51</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E17" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C17,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C17,'Price List'!$C$3:$C$23,0))</f>
         <v>392850</v>
       </c>
       <c r="G17" s="20" t="n">
@@ -10657,15 +11030,15 @@
         <v>392850</v>
       </c>
       <c r="H17" s="34" t="n">
-        <f aca="false">E17*INDEX('Price List'!$K$3:$K$20,MATCH($C17,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E17*INDEX('Price List'!$K$3:$K$23,MATCH($C17,'Price List'!$C$3:$C$23,0))</f>
         <v>14</v>
       </c>
       <c r="I17" s="34" t="n">
-        <f aca="false">E17*INDEX('Price List'!$L$3:$L$20,MATCH($C17,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E17*INDEX('Price List'!$L$3:$L$23,MATCH($C17,'Price List'!$C$3:$C$23,0))</f>
         <v>10</v>
       </c>
       <c r="J17" s="34" t="n">
-        <f aca="false">E17*INDEX('Price List'!$M$3:$M$20,MATCH($C17,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E17*INDEX('Price List'!$M$3:$M$23,MATCH($C17,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K17" s="34" t="n">
@@ -10673,15 +11046,15 @@
         <v>10</v>
       </c>
       <c r="L17" s="34" t="n">
-        <f aca="false">E17*INDEX('Price List'!$O$3:$O$20,MATCH($C17,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E17*INDEX('Price List'!$O$3:$O$23,MATCH($C17,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M17" s="34" t="n">
-        <f aca="false">E17*INDEX('Price List'!$P$3:$P$20,MATCH($C17,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E17*INDEX('Price List'!$P$3:$P$23,MATCH($C17,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="N17" s="34" t="n">
-        <f aca="false">E17*INDEX('Price List'!$Q$3:$Q$20,MATCH($C17,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E17*INDEX('Price List'!$Q$3:$Q$23,MATCH($C17,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O17" s="34" t="n">
@@ -10699,19 +11072,19 @@
         <v>12</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C18" s="32" t="s">
         <v>62</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E18" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C18,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C18,'Price List'!$C$3:$C$23,0))</f>
         <v>90800</v>
       </c>
       <c r="G18" s="20" t="n">
@@ -10719,15 +11092,15 @@
         <v>90800</v>
       </c>
       <c r="H18" s="34" t="n">
-        <f aca="false">E18*INDEX('Price List'!$K$3:$K$20,MATCH($C18,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E18*INDEX('Price List'!$K$3:$K$23,MATCH($C18,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I18" s="34" t="n">
-        <f aca="false">E18*INDEX('Price List'!$L$3:$L$20,MATCH($C18,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E18*INDEX('Price List'!$L$3:$L$23,MATCH($C18,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J18" s="34" t="n">
-        <f aca="false">E18*INDEX('Price List'!$M$3:$M$20,MATCH($C18,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E18*INDEX('Price List'!$M$3:$M$23,MATCH($C18,'Price List'!$C$3:$C$23,0))</f>
         <v>16</v>
       </c>
       <c r="K18" s="34" t="n">
@@ -10735,15 +11108,15 @@
         <v>16</v>
       </c>
       <c r="L18" s="34" t="n">
-        <f aca="false">E18*INDEX('Price List'!$O$3:$O$20,MATCH($C18,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E18*INDEX('Price List'!$O$3:$O$23,MATCH($C18,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M18" s="34" t="n">
-        <f aca="false">E18*INDEX('Price List'!$P$3:$P$20,MATCH($C18,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E18*INDEX('Price List'!$P$3:$P$23,MATCH($C18,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N18" s="34" t="n">
-        <f aca="false">E18*INDEX('Price List'!$Q$3:$Q$20,MATCH($C18,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E18*INDEX('Price List'!$Q$3:$Q$23,MATCH($C18,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O18" s="34" t="n">
@@ -10761,19 +11134,19 @@
         <v>12</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C19" s="32" t="s">
         <v>80</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="E19" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C19,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C19,'Price List'!$C$3:$C$23,0))</f>
         <v>138400</v>
       </c>
       <c r="G19" s="20" t="n">
@@ -10781,15 +11154,15 @@
         <v>138400</v>
       </c>
       <c r="H19" s="34" t="n">
-        <f aca="false">E19*INDEX('Price List'!$K$3:$K$20,MATCH($C19,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E19*INDEX('Price List'!$K$3:$K$23,MATCH($C19,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I19" s="34" t="n">
-        <f aca="false">E19*INDEX('Price List'!$L$3:$L$20,MATCH($C19,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E19*INDEX('Price List'!$L$3:$L$23,MATCH($C19,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J19" s="34" t="n">
-        <f aca="false">E19*INDEX('Price List'!$M$3:$M$20,MATCH($C19,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E19*INDEX('Price List'!$M$3:$M$23,MATCH($C19,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K19" s="34" t="n">
@@ -10797,15 +11170,15 @@
         <v>0</v>
       </c>
       <c r="L19" s="34" t="n">
-        <f aca="false">E19*INDEX('Price List'!$O$3:$O$20,MATCH($C19,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E19*INDEX('Price List'!$O$3:$O$23,MATCH($C19,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="M19" s="34" t="n">
-        <f aca="false">E19*INDEX('Price List'!$P$3:$P$20,MATCH($C19,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E19*INDEX('Price List'!$P$3:$P$23,MATCH($C19,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N19" s="34" t="n">
-        <f aca="false">E19*INDEX('Price List'!$Q$3:$Q$20,MATCH($C19,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E19*INDEX('Price List'!$Q$3:$Q$23,MATCH($C19,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O19" s="34" t="n">
@@ -10823,13 +11196,13 @@
         <v>12</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C20" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E20" s="36"/>
       <c r="F20" s="36"/>
@@ -10880,19 +11253,19 @@
         <v>12</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C21" s="32" t="s">
         <v>56</v>
       </c>
       <c r="D21" s="32" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="E21" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C21,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C21,'Price List'!$C$3:$C$23,0))</f>
         <v>417600</v>
       </c>
       <c r="G21" s="20" t="n">
@@ -10900,15 +11273,15 @@
         <v>417600</v>
       </c>
       <c r="H21" s="34" t="n">
-        <f aca="false">E21*INDEX('Price List'!$K$3:$K$20,MATCH($C21,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E21*INDEX('Price List'!$K$3:$K$23,MATCH($C21,'Price List'!$C$3:$C$23,0))</f>
         <v>24</v>
       </c>
       <c r="I21" s="34" t="n">
-        <f aca="false">E21*INDEX('Price List'!$L$3:$L$20,MATCH($C21,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E21*INDEX('Price List'!$L$3:$L$23,MATCH($C21,'Price List'!$C$3:$C$23,0))</f>
         <v>16</v>
       </c>
       <c r="J21" s="34" t="n">
-        <f aca="false">E21*INDEX('Price List'!$M$3:$M$20,MATCH($C21,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E21*INDEX('Price List'!$M$3:$M$23,MATCH($C21,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K21" s="34" t="n">
@@ -10916,15 +11289,15 @@
         <v>16</v>
       </c>
       <c r="L21" s="34" t="n">
-        <f aca="false">E21*INDEX('Price List'!$O$3:$O$20,MATCH($C21,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E21*INDEX('Price List'!$O$3:$O$23,MATCH($C21,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M21" s="34" t="n">
-        <f aca="false">E21*INDEX('Price List'!$P$3:$P$20,MATCH($C21,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E21*INDEX('Price List'!$P$3:$P$23,MATCH($C21,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="N21" s="34" t="n">
-        <f aca="false">E21*INDEX('Price List'!$Q$3:$Q$20,MATCH($C21,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E21*INDEX('Price List'!$Q$3:$Q$23,MATCH($C21,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O21" s="34" t="n">
@@ -10942,19 +11315,19 @@
         <v>12</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C22" s="32" t="s">
         <v>80</v>
       </c>
       <c r="D22" s="32" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="E22" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C22,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C22,'Price List'!$C$3:$C$23,0))</f>
         <v>138400</v>
       </c>
       <c r="G22" s="20" t="n">
@@ -10962,15 +11335,15 @@
         <v>138400</v>
       </c>
       <c r="H22" s="34" t="n">
-        <f aca="false">E22*INDEX('Price List'!$K$3:$K$20,MATCH($C22,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E22*INDEX('Price List'!$K$3:$K$23,MATCH($C22,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I22" s="34" t="n">
-        <f aca="false">E22*INDEX('Price List'!$L$3:$L$20,MATCH($C22,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E22*INDEX('Price List'!$L$3:$L$23,MATCH($C22,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J22" s="34" t="n">
-        <f aca="false">E22*INDEX('Price List'!$M$3:$M$20,MATCH($C22,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E22*INDEX('Price List'!$M$3:$M$23,MATCH($C22,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K22" s="34" t="n">
@@ -10978,15 +11351,15 @@
         <v>0</v>
       </c>
       <c r="L22" s="34" t="n">
-        <f aca="false">E22*INDEX('Price List'!$O$3:$O$20,MATCH($C22,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E22*INDEX('Price List'!$O$3:$O$23,MATCH($C22,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="M22" s="34" t="n">
-        <f aca="false">E22*INDEX('Price List'!$P$3:$P$20,MATCH($C22,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E22*INDEX('Price List'!$P$3:$P$23,MATCH($C22,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N22" s="34" t="n">
-        <f aca="false">E22*INDEX('Price List'!$Q$3:$Q$20,MATCH($C22,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E22*INDEX('Price List'!$Q$3:$Q$23,MATCH($C22,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O22" s="34" t="n">
@@ -11004,13 +11377,13 @@
         <v>12</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C23" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D23" s="36" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="E23" s="36"/>
       <c r="F23" s="36"/>
@@ -11061,19 +11434,19 @@
         <v>12</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C24" s="32" t="s">
         <v>57</v>
       </c>
       <c r="D24" s="32" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E24" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C24,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C24,'Price List'!$C$3:$C$23,0))</f>
         <v>406350</v>
       </c>
       <c r="G24" s="20" t="n">
@@ -11081,15 +11454,15 @@
         <v>406350</v>
       </c>
       <c r="H24" s="34" t="n">
-        <f aca="false">E24*INDEX('Price List'!$K$3:$K$20,MATCH($C24,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E24*INDEX('Price List'!$K$3:$K$23,MATCH($C24,'Price List'!$C$3:$C$23,0))</f>
         <v>24</v>
       </c>
       <c r="I24" s="34" t="n">
-        <f aca="false">E24*INDEX('Price List'!$L$3:$L$20,MATCH($C24,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E24*INDEX('Price List'!$L$3:$L$23,MATCH($C24,'Price List'!$C$3:$C$23,0))</f>
         <v>4</v>
       </c>
       <c r="J24" s="34" t="n">
-        <f aca="false">E24*INDEX('Price List'!$M$3:$M$20,MATCH($C24,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E24*INDEX('Price List'!$M$3:$M$23,MATCH($C24,'Price List'!$C$3:$C$23,0))</f>
         <v>12</v>
       </c>
       <c r="K24" s="34" t="n">
@@ -11097,15 +11470,15 @@
         <v>16</v>
       </c>
       <c r="L24" s="34" t="n">
-        <f aca="false">E24*INDEX('Price List'!$O$3:$O$20,MATCH($C24,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E24*INDEX('Price List'!$O$3:$O$23,MATCH($C24,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M24" s="34" t="n">
-        <f aca="false">E24*INDEX('Price List'!$P$3:$P$20,MATCH($C24,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E24*INDEX('Price List'!$P$3:$P$23,MATCH($C24,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="N24" s="34" t="n">
-        <f aca="false">E24*INDEX('Price List'!$Q$3:$Q$20,MATCH($C24,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E24*INDEX('Price List'!$Q$3:$Q$23,MATCH($C24,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O24" s="34" t="n">
@@ -11123,19 +11496,19 @@
         <v>12</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C25" s="32" t="s">
         <v>80</v>
       </c>
       <c r="D25" s="32" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="E25" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C25,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C25,'Price List'!$C$3:$C$23,0))</f>
         <v>138400</v>
       </c>
       <c r="G25" s="20" t="n">
@@ -11143,15 +11516,15 @@
         <v>138400</v>
       </c>
       <c r="H25" s="34" t="n">
-        <f aca="false">E25*INDEX('Price List'!$K$3:$K$20,MATCH($C25,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E25*INDEX('Price List'!$K$3:$K$23,MATCH($C25,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I25" s="34" t="n">
-        <f aca="false">E25*INDEX('Price List'!$L$3:$L$20,MATCH($C25,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E25*INDEX('Price List'!$L$3:$L$23,MATCH($C25,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J25" s="34" t="n">
-        <f aca="false">E25*INDEX('Price List'!$M$3:$M$20,MATCH($C25,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E25*INDEX('Price List'!$M$3:$M$23,MATCH($C25,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K25" s="34" t="n">
@@ -11159,15 +11532,15 @@
         <v>0</v>
       </c>
       <c r="L25" s="34" t="n">
-        <f aca="false">E25*INDEX('Price List'!$O$3:$O$20,MATCH($C25,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E25*INDEX('Price List'!$O$3:$O$23,MATCH($C25,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="M25" s="34" t="n">
-        <f aca="false">E25*INDEX('Price List'!$P$3:$P$20,MATCH($C25,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E25*INDEX('Price List'!$P$3:$P$23,MATCH($C25,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N25" s="34" t="n">
-        <f aca="false">E25*INDEX('Price List'!$Q$3:$Q$20,MATCH($C25,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E25*INDEX('Price List'!$Q$3:$Q$23,MATCH($C25,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O25" s="34" t="n">
@@ -11185,13 +11558,13 @@
         <v>12</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C26" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E26" s="36"/>
       <c r="F26" s="36"/>
@@ -11239,7 +11612,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="28" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B28" s="28"/>
       <c r="C28" s="28"/>
@@ -11263,11 +11636,11 @@
         <v>14</v>
       </c>
       <c r="B29" s="30" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C29" s="30"/>
       <c r="D29" s="31" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="E29" s="30"/>
       <c r="F29" s="30"/>
@@ -11298,19 +11671,19 @@
         <v>14</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C30" s="32" t="s">
         <v>51</v>
       </c>
       <c r="D30" s="32" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="E30" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C30,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C30,'Price List'!$C$3:$C$23,0))</f>
         <v>392850</v>
       </c>
       <c r="G30" s="20" t="n">
@@ -11318,15 +11691,15 @@
         <v>392850</v>
       </c>
       <c r="H30" s="34" t="n">
-        <f aca="false">E30*INDEX('Price List'!$K$3:$K$20,MATCH($C30,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E30*INDEX('Price List'!$K$3:$K$23,MATCH($C30,'Price List'!$C$3:$C$23,0))</f>
         <v>14</v>
       </c>
       <c r="I30" s="34" t="n">
-        <f aca="false">E30*INDEX('Price List'!$L$3:$L$20,MATCH($C30,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E30*INDEX('Price List'!$L$3:$L$23,MATCH($C30,'Price List'!$C$3:$C$23,0))</f>
         <v>10</v>
       </c>
       <c r="J30" s="34" t="n">
-        <f aca="false">E30*INDEX('Price List'!$M$3:$M$20,MATCH($C30,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E30*INDEX('Price List'!$M$3:$M$23,MATCH($C30,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K30" s="34" t="n">
@@ -11334,15 +11707,15 @@
         <v>10</v>
       </c>
       <c r="L30" s="34" t="n">
-        <f aca="false">E30*INDEX('Price List'!$O$3:$O$20,MATCH($C30,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E30*INDEX('Price List'!$O$3:$O$23,MATCH($C30,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M30" s="34" t="n">
-        <f aca="false">E30*INDEX('Price List'!$P$3:$P$20,MATCH($C30,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E30*INDEX('Price List'!$P$3:$P$23,MATCH($C30,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="N30" s="34" t="n">
-        <f aca="false">E30*INDEX('Price List'!$Q$3:$Q$20,MATCH($C30,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E30*INDEX('Price List'!$Q$3:$Q$23,MATCH($C30,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O30" s="34" t="n">
@@ -11360,19 +11733,19 @@
         <v>14</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C31" s="32" t="s">
         <v>68</v>
       </c>
       <c r="D31" s="32" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="E31" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C31,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C31,'Price List'!$C$3:$C$23,0))</f>
         <v>64400</v>
       </c>
       <c r="G31" s="20" t="n">
@@ -11380,15 +11753,15 @@
         <v>64400</v>
       </c>
       <c r="H31" s="34" t="n">
-        <f aca="false">E31*INDEX('Price List'!$K$3:$K$20,MATCH($C31,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E31*INDEX('Price List'!$K$3:$K$23,MATCH($C31,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I31" s="34" t="n">
-        <f aca="false">E31*INDEX('Price List'!$L$3:$L$20,MATCH($C31,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E31*INDEX('Price List'!$L$3:$L$23,MATCH($C31,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J31" s="34" t="n">
-        <f aca="false">E31*INDEX('Price List'!$M$3:$M$20,MATCH($C31,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E31*INDEX('Price List'!$M$3:$M$23,MATCH($C31,'Price List'!$C$3:$C$23,0))</f>
         <v>8</v>
       </c>
       <c r="K31" s="34" t="n">
@@ -11396,15 +11769,15 @@
         <v>8</v>
       </c>
       <c r="L31" s="34" t="n">
-        <f aca="false">E31*INDEX('Price List'!$O$3:$O$20,MATCH($C31,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E31*INDEX('Price List'!$O$3:$O$23,MATCH($C31,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M31" s="34" t="n">
-        <f aca="false">E31*INDEX('Price List'!$P$3:$P$20,MATCH($C31,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E31*INDEX('Price List'!$P$3:$P$23,MATCH($C31,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N31" s="34" t="n">
-        <f aca="false">E31*INDEX('Price List'!$Q$3:$Q$20,MATCH($C31,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E31*INDEX('Price List'!$Q$3:$Q$23,MATCH($C31,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O31" s="34" t="n">
@@ -11422,19 +11795,19 @@
         <v>14</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C32" s="32" t="s">
         <v>80</v>
       </c>
       <c r="D32" s="32" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E32" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C32,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C32,'Price List'!$C$3:$C$23,0))</f>
         <v>138400</v>
       </c>
       <c r="G32" s="20" t="n">
@@ -11442,15 +11815,15 @@
         <v>138400</v>
       </c>
       <c r="H32" s="34" t="n">
-        <f aca="false">E32*INDEX('Price List'!$K$3:$K$20,MATCH($C32,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E32*INDEX('Price List'!$K$3:$K$23,MATCH($C32,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I32" s="34" t="n">
-        <f aca="false">E32*INDEX('Price List'!$L$3:$L$20,MATCH($C32,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E32*INDEX('Price List'!$L$3:$L$23,MATCH($C32,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J32" s="34" t="n">
-        <f aca="false">E32*INDEX('Price List'!$M$3:$M$20,MATCH($C32,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E32*INDEX('Price List'!$M$3:$M$23,MATCH($C32,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K32" s="34" t="n">
@@ -11458,15 +11831,15 @@
         <v>0</v>
       </c>
       <c r="L32" s="34" t="n">
-        <f aca="false">E32*INDEX('Price List'!$O$3:$O$20,MATCH($C32,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E32*INDEX('Price List'!$O$3:$O$23,MATCH($C32,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="M32" s="34" t="n">
-        <f aca="false">E32*INDEX('Price List'!$P$3:$P$20,MATCH($C32,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E32*INDEX('Price List'!$P$3:$P$23,MATCH($C32,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N32" s="34" t="n">
-        <f aca="false">E32*INDEX('Price List'!$Q$3:$Q$20,MATCH($C32,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E32*INDEX('Price List'!$Q$3:$Q$23,MATCH($C32,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O32" s="34" t="n">
@@ -11484,13 +11857,13 @@
         <v>14</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C33" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D33" s="36" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E33" s="36"/>
       <c r="F33" s="36"/>
@@ -11541,19 +11914,19 @@
         <v>14</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C34" s="32" t="s">
         <v>51</v>
       </c>
       <c r="D34" s="32" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="E34" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C34,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C34,'Price List'!$C$3:$C$23,0))</f>
         <v>392850</v>
       </c>
       <c r="G34" s="20" t="n">
@@ -11561,15 +11934,15 @@
         <v>392850</v>
       </c>
       <c r="H34" s="34" t="n">
-        <f aca="false">E34*INDEX('Price List'!$K$3:$K$20,MATCH($C34,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E34*INDEX('Price List'!$K$3:$K$23,MATCH($C34,'Price List'!$C$3:$C$23,0))</f>
         <v>14</v>
       </c>
       <c r="I34" s="34" t="n">
-        <f aca="false">E34*INDEX('Price List'!$L$3:$L$20,MATCH($C34,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E34*INDEX('Price List'!$L$3:$L$23,MATCH($C34,'Price List'!$C$3:$C$23,0))</f>
         <v>10</v>
       </c>
       <c r="J34" s="34" t="n">
-        <f aca="false">E34*INDEX('Price List'!$M$3:$M$20,MATCH($C34,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E34*INDEX('Price List'!$M$3:$M$23,MATCH($C34,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K34" s="34" t="n">
@@ -11577,15 +11950,15 @@
         <v>10</v>
       </c>
       <c r="L34" s="34" t="n">
-        <f aca="false">E34*INDEX('Price List'!$O$3:$O$20,MATCH($C34,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E34*INDEX('Price List'!$O$3:$O$23,MATCH($C34,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M34" s="34" t="n">
-        <f aca="false">E34*INDEX('Price List'!$P$3:$P$20,MATCH($C34,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E34*INDEX('Price List'!$P$3:$P$23,MATCH($C34,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="N34" s="34" t="n">
-        <f aca="false">E34*INDEX('Price List'!$Q$3:$Q$20,MATCH($C34,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E34*INDEX('Price List'!$Q$3:$Q$23,MATCH($C34,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O34" s="34" t="n">
@@ -11603,19 +11976,19 @@
         <v>14</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C35" s="32" t="s">
         <v>80</v>
       </c>
       <c r="D35" s="32" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E35" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C35,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C35,'Price List'!$C$3:$C$23,0))</f>
         <v>138400</v>
       </c>
       <c r="G35" s="20" t="n">
@@ -11623,15 +11996,15 @@
         <v>138400</v>
       </c>
       <c r="H35" s="34" t="n">
-        <f aca="false">E35*INDEX('Price List'!$K$3:$K$20,MATCH($C35,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E35*INDEX('Price List'!$K$3:$K$23,MATCH($C35,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I35" s="34" t="n">
-        <f aca="false">E35*INDEX('Price List'!$L$3:$L$20,MATCH($C35,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E35*INDEX('Price List'!$L$3:$L$23,MATCH($C35,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J35" s="34" t="n">
-        <f aca="false">E35*INDEX('Price List'!$M$3:$M$20,MATCH($C35,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E35*INDEX('Price List'!$M$3:$M$23,MATCH($C35,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K35" s="34" t="n">
@@ -11639,15 +12012,15 @@
         <v>0</v>
       </c>
       <c r="L35" s="34" t="n">
-        <f aca="false">E35*INDEX('Price List'!$O$3:$O$20,MATCH($C35,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E35*INDEX('Price List'!$O$3:$O$23,MATCH($C35,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="M35" s="34" t="n">
-        <f aca="false">E35*INDEX('Price List'!$P$3:$P$20,MATCH($C35,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E35*INDEX('Price List'!$P$3:$P$23,MATCH($C35,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N35" s="34" t="n">
-        <f aca="false">E35*INDEX('Price List'!$Q$3:$Q$20,MATCH($C35,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E35*INDEX('Price List'!$Q$3:$Q$23,MATCH($C35,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O35" s="34" t="n">
@@ -11665,13 +12038,13 @@
         <v>14</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C36" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D36" s="36" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="E36" s="36"/>
       <c r="F36" s="36"/>
@@ -11722,19 +12095,19 @@
         <v>14</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C37" s="32" t="s">
         <v>53</v>
       </c>
       <c r="D37" s="32" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="E37" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C37,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C37,'Price List'!$C$3:$C$23,0))</f>
         <v>384750</v>
       </c>
       <c r="G37" s="20" t="n">
@@ -11742,15 +12115,15 @@
         <v>384750</v>
       </c>
       <c r="H37" s="34" t="n">
-        <f aca="false">E37*INDEX('Price List'!$K$3:$K$20,MATCH($C37,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E37*INDEX('Price List'!$K$3:$K$23,MATCH($C37,'Price List'!$C$3:$C$23,0))</f>
         <v>14</v>
       </c>
       <c r="I37" s="34" t="n">
-        <f aca="false">E37*INDEX('Price List'!$L$3:$L$20,MATCH($C37,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E37*INDEX('Price List'!$L$3:$L$23,MATCH($C37,'Price List'!$C$3:$C$23,0))</f>
         <v>4</v>
       </c>
       <c r="J37" s="34" t="n">
-        <f aca="false">E37*INDEX('Price List'!$M$3:$M$20,MATCH($C37,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E37*INDEX('Price List'!$M$3:$M$23,MATCH($C37,'Price List'!$C$3:$C$23,0))</f>
         <v>6</v>
       </c>
       <c r="K37" s="34" t="n">
@@ -11758,15 +12131,15 @@
         <v>10</v>
       </c>
       <c r="L37" s="34" t="n">
-        <f aca="false">E37*INDEX('Price List'!$O$3:$O$20,MATCH($C37,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E37*INDEX('Price List'!$O$3:$O$23,MATCH($C37,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M37" s="34" t="n">
-        <f aca="false">E37*INDEX('Price List'!$P$3:$P$20,MATCH($C37,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E37*INDEX('Price List'!$P$3:$P$23,MATCH($C37,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="N37" s="34" t="n">
-        <f aca="false">E37*INDEX('Price List'!$Q$3:$Q$20,MATCH($C37,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E37*INDEX('Price List'!$Q$3:$Q$23,MATCH($C37,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O37" s="34" t="n">
@@ -11784,19 +12157,19 @@
         <v>14</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C38" s="32" t="s">
         <v>80</v>
       </c>
       <c r="D38" s="32" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E38" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C38,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C38,'Price List'!$C$3:$C$23,0))</f>
         <v>138400</v>
       </c>
       <c r="G38" s="20" t="n">
@@ -11804,15 +12177,15 @@
         <v>138400</v>
       </c>
       <c r="H38" s="34" t="n">
-        <f aca="false">E38*INDEX('Price List'!$K$3:$K$20,MATCH($C38,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E38*INDEX('Price List'!$K$3:$K$23,MATCH($C38,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I38" s="34" t="n">
-        <f aca="false">E38*INDEX('Price List'!$L$3:$L$20,MATCH($C38,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E38*INDEX('Price List'!$L$3:$L$23,MATCH($C38,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J38" s="34" t="n">
-        <f aca="false">E38*INDEX('Price List'!$M$3:$M$20,MATCH($C38,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E38*INDEX('Price List'!$M$3:$M$23,MATCH($C38,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K38" s="34" t="n">
@@ -11820,15 +12193,15 @@
         <v>0</v>
       </c>
       <c r="L38" s="34" t="n">
-        <f aca="false">E38*INDEX('Price List'!$O$3:$O$20,MATCH($C38,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E38*INDEX('Price List'!$O$3:$O$23,MATCH($C38,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="M38" s="34" t="n">
-        <f aca="false">E38*INDEX('Price List'!$P$3:$P$20,MATCH($C38,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E38*INDEX('Price List'!$P$3:$P$23,MATCH($C38,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N38" s="34" t="n">
-        <f aca="false">E38*INDEX('Price List'!$Q$3:$Q$20,MATCH($C38,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E38*INDEX('Price List'!$Q$3:$Q$23,MATCH($C38,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O38" s="34" t="n">
@@ -11846,13 +12219,13 @@
         <v>14</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C39" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D39" s="36" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E39" s="36"/>
       <c r="F39" s="36"/>
@@ -11900,7 +12273,7 @@
     </row>
     <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="28" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B41" s="28"/>
       <c r="C41" s="28"/>
@@ -11924,11 +12297,11 @@
         <v>16</v>
       </c>
       <c r="B42" s="30" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C42" s="30"/>
       <c r="D42" s="31" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E42" s="30"/>
       <c r="F42" s="30"/>
@@ -11959,19 +12332,19 @@
         <v>16</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C43" s="32" t="s">
         <v>48</v>
       </c>
       <c r="D43" s="32" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E43" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C43,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C43,'Price List'!$C$3:$C$23,0))</f>
         <v>398700</v>
       </c>
       <c r="G43" s="20" t="n">
@@ -11979,15 +12352,15 @@
         <v>398700</v>
       </c>
       <c r="H43" s="34" t="n">
-        <f aca="false">E43*INDEX('Price List'!$K$3:$K$20,MATCH($C43,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E43*INDEX('Price List'!$K$3:$K$23,MATCH($C43,'Price List'!$C$3:$C$23,0))</f>
         <v>14</v>
       </c>
       <c r="I43" s="34" t="n">
-        <f aca="false">E43*INDEX('Price List'!$L$3:$L$20,MATCH($C43,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E43*INDEX('Price List'!$L$3:$L$23,MATCH($C43,'Price List'!$C$3:$C$23,0))</f>
         <v>10</v>
       </c>
       <c r="J43" s="34" t="n">
-        <f aca="false">E43*INDEX('Price List'!$M$3:$M$20,MATCH($C43,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E43*INDEX('Price List'!$M$3:$M$23,MATCH($C43,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K43" s="34" t="n">
@@ -11995,15 +12368,15 @@
         <v>10</v>
       </c>
       <c r="L43" s="34" t="n">
-        <f aca="false">E43*INDEX('Price List'!$O$3:$O$20,MATCH($C43,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E43*INDEX('Price List'!$O$3:$O$23,MATCH($C43,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M43" s="34" t="n">
-        <f aca="false">E43*INDEX('Price List'!$P$3:$P$20,MATCH($C43,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E43*INDEX('Price List'!$P$3:$P$23,MATCH($C43,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="N43" s="34" t="n">
-        <f aca="false">E43*INDEX('Price List'!$Q$3:$Q$20,MATCH($C43,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E43*INDEX('Price List'!$Q$3:$Q$23,MATCH($C43,'Price List'!$C$3:$C$23,0))</f>
         <v>1</v>
       </c>
       <c r="O43" s="34" t="n">
@@ -12021,19 +12394,19 @@
         <v>16</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C44" s="32" t="s">
         <v>58</v>
       </c>
       <c r="D44" s="32" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="E44" s="33" t="n">
         <v>6</v>
       </c>
       <c r="F44" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C44,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C44,'Price List'!$C$3:$C$23,0))</f>
         <v>91200</v>
       </c>
       <c r="G44" s="20" t="n">
@@ -12041,15 +12414,15 @@
         <v>547200</v>
       </c>
       <c r="H44" s="34" t="n">
-        <f aca="false">E44*INDEX('Price List'!$K$3:$K$20,MATCH($C44,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E44*INDEX('Price List'!$K$3:$K$23,MATCH($C44,'Price List'!$C$3:$C$23,0))</f>
         <v>96</v>
       </c>
       <c r="I44" s="34" t="n">
-        <f aca="false">E44*INDEX('Price List'!$L$3:$L$20,MATCH($C44,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E44*INDEX('Price List'!$L$3:$L$23,MATCH($C44,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J44" s="34" t="n">
-        <f aca="false">E44*INDEX('Price List'!$M$3:$M$20,MATCH($C44,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E44*INDEX('Price List'!$M$3:$M$23,MATCH($C44,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K44" s="34" t="n">
@@ -12057,15 +12430,15 @@
         <v>0</v>
       </c>
       <c r="L44" s="34" t="n">
-        <f aca="false">E44*INDEX('Price List'!$O$3:$O$20,MATCH($C44,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E44*INDEX('Price List'!$O$3:$O$23,MATCH($C44,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M44" s="34" t="n">
-        <f aca="false">E44*INDEX('Price List'!$P$3:$P$20,MATCH($C44,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E44*INDEX('Price List'!$P$3:$P$23,MATCH($C44,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N44" s="34" t="n">
-        <f aca="false">E44*INDEX('Price List'!$Q$3:$Q$20,MATCH($C44,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E44*INDEX('Price List'!$Q$3:$Q$23,MATCH($C44,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O44" s="34" t="n">
@@ -12083,19 +12456,19 @@
         <v>16</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C45" s="32" t="s">
         <v>62</v>
       </c>
       <c r="D45" s="32" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="E45" s="33" t="n">
         <v>4</v>
       </c>
       <c r="F45" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C45,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C45,'Price List'!$C$3:$C$23,0))</f>
         <v>90800</v>
       </c>
       <c r="G45" s="20" t="n">
@@ -12103,15 +12476,15 @@
         <v>363200</v>
       </c>
       <c r="H45" s="34" t="n">
-        <f aca="false">E45*INDEX('Price List'!$K$3:$K$20,MATCH($C45,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E45*INDEX('Price List'!$K$3:$K$23,MATCH($C45,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I45" s="34" t="n">
-        <f aca="false">E45*INDEX('Price List'!$L$3:$L$20,MATCH($C45,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E45*INDEX('Price List'!$L$3:$L$23,MATCH($C45,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J45" s="34" t="n">
-        <f aca="false">E45*INDEX('Price List'!$M$3:$M$20,MATCH($C45,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E45*INDEX('Price List'!$M$3:$M$23,MATCH($C45,'Price List'!$C$3:$C$23,0))</f>
         <v>64</v>
       </c>
       <c r="K45" s="34" t="n">
@@ -12119,15 +12492,15 @@
         <v>64</v>
       </c>
       <c r="L45" s="34" t="n">
-        <f aca="false">E45*INDEX('Price List'!$O$3:$O$20,MATCH($C45,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E45*INDEX('Price List'!$O$3:$O$23,MATCH($C45,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M45" s="34" t="n">
-        <f aca="false">E45*INDEX('Price List'!$P$3:$P$20,MATCH($C45,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E45*INDEX('Price List'!$P$3:$P$23,MATCH($C45,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N45" s="34" t="n">
-        <f aca="false">E45*INDEX('Price List'!$Q$3:$Q$20,MATCH($C45,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E45*INDEX('Price List'!$Q$3:$Q$23,MATCH($C45,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O45" s="34" t="n">
@@ -12145,19 +12518,19 @@
         <v>16</v>
       </c>
       <c r="B46" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C46" s="32" t="s">
         <v>82</v>
       </c>
       <c r="D46" s="32" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E46" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F46" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C46,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C46,'Price List'!$C$3:$C$23,0))</f>
         <v>140400</v>
       </c>
       <c r="G46" s="20" t="n">
@@ -12165,15 +12538,15 @@
         <v>140400</v>
       </c>
       <c r="H46" s="34" t="n">
-        <f aca="false">E46*INDEX('Price List'!$K$3:$K$20,MATCH($C46,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E46*INDEX('Price List'!$K$3:$K$23,MATCH($C46,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I46" s="34" t="n">
-        <f aca="false">E46*INDEX('Price List'!$L$3:$L$20,MATCH($C46,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E46*INDEX('Price List'!$L$3:$L$23,MATCH($C46,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J46" s="34" t="n">
-        <f aca="false">E46*INDEX('Price List'!$M$3:$M$20,MATCH($C46,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E46*INDEX('Price List'!$M$3:$M$23,MATCH($C46,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K46" s="34" t="n">
@@ -12181,15 +12554,15 @@
         <v>0</v>
       </c>
       <c r="L46" s="34" t="n">
-        <f aca="false">E46*INDEX('Price List'!$O$3:$O$20,MATCH($C46,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E46*INDEX('Price List'!$O$3:$O$23,MATCH($C46,'Price List'!$C$3:$C$23,0))</f>
         <v>4</v>
       </c>
       <c r="M46" s="34" t="n">
-        <f aca="false">E46*INDEX('Price List'!$P$3:$P$20,MATCH($C46,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E46*INDEX('Price List'!$P$3:$P$23,MATCH($C46,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N46" s="34" t="n">
-        <f aca="false">E46*INDEX('Price List'!$Q$3:$Q$20,MATCH($C46,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E46*INDEX('Price List'!$Q$3:$Q$23,MATCH($C46,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O46" s="34" t="n">
@@ -12207,13 +12580,13 @@
         <v>16</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C47" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D47" s="36" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E47" s="36"/>
       <c r="F47" s="36"/>
@@ -12264,19 +12637,19 @@
         <v>16</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C48" s="32" t="s">
         <v>48</v>
       </c>
       <c r="D48" s="32" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E48" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F48" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C48,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C48,'Price List'!$C$3:$C$23,0))</f>
         <v>398700</v>
       </c>
       <c r="G48" s="20" t="n">
@@ -12284,15 +12657,15 @@
         <v>398700</v>
       </c>
       <c r="H48" s="34" t="n">
-        <f aca="false">E48*INDEX('Price List'!$K$3:$K$20,MATCH($C48,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E48*INDEX('Price List'!$K$3:$K$23,MATCH($C48,'Price List'!$C$3:$C$23,0))</f>
         <v>14</v>
       </c>
       <c r="I48" s="34" t="n">
-        <f aca="false">E48*INDEX('Price List'!$L$3:$L$20,MATCH($C48,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E48*INDEX('Price List'!$L$3:$L$23,MATCH($C48,'Price List'!$C$3:$C$23,0))</f>
         <v>10</v>
       </c>
       <c r="J48" s="34" t="n">
-        <f aca="false">E48*INDEX('Price List'!$M$3:$M$20,MATCH($C48,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E48*INDEX('Price List'!$M$3:$M$23,MATCH($C48,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K48" s="34" t="n">
@@ -12300,15 +12673,15 @@
         <v>10</v>
       </c>
       <c r="L48" s="34" t="n">
-        <f aca="false">E48*INDEX('Price List'!$O$3:$O$20,MATCH($C48,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E48*INDEX('Price List'!$O$3:$O$23,MATCH($C48,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M48" s="34" t="n">
-        <f aca="false">E48*INDEX('Price List'!$P$3:$P$20,MATCH($C48,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E48*INDEX('Price List'!$P$3:$P$23,MATCH($C48,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="N48" s="34" t="n">
-        <f aca="false">E48*INDEX('Price List'!$Q$3:$Q$20,MATCH($C48,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E48*INDEX('Price List'!$Q$3:$Q$23,MATCH($C48,'Price List'!$C$3:$C$23,0))</f>
         <v>1</v>
       </c>
       <c r="O48" s="34" t="n">
@@ -12326,19 +12699,19 @@
         <v>16</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C49" s="32" t="s">
         <v>58</v>
       </c>
       <c r="D49" s="32" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="E49" s="33" t="n">
         <v>6</v>
       </c>
       <c r="F49" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C49,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C49,'Price List'!$C$3:$C$23,0))</f>
         <v>91200</v>
       </c>
       <c r="G49" s="20" t="n">
@@ -12346,15 +12719,15 @@
         <v>547200</v>
       </c>
       <c r="H49" s="34" t="n">
-        <f aca="false">E49*INDEX('Price List'!$K$3:$K$20,MATCH($C49,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E49*INDEX('Price List'!$K$3:$K$23,MATCH($C49,'Price List'!$C$3:$C$23,0))</f>
         <v>96</v>
       </c>
       <c r="I49" s="34" t="n">
-        <f aca="false">E49*INDEX('Price List'!$L$3:$L$20,MATCH($C49,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E49*INDEX('Price List'!$L$3:$L$23,MATCH($C49,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J49" s="34" t="n">
-        <f aca="false">E49*INDEX('Price List'!$M$3:$M$20,MATCH($C49,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E49*INDEX('Price List'!$M$3:$M$23,MATCH($C49,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K49" s="34" t="n">
@@ -12362,15 +12735,15 @@
         <v>0</v>
       </c>
       <c r="L49" s="34" t="n">
-        <f aca="false">E49*INDEX('Price List'!$O$3:$O$20,MATCH($C49,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E49*INDEX('Price List'!$O$3:$O$23,MATCH($C49,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M49" s="34" t="n">
-        <f aca="false">E49*INDEX('Price List'!$P$3:$P$20,MATCH($C49,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E49*INDEX('Price List'!$P$3:$P$23,MATCH($C49,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N49" s="34" t="n">
-        <f aca="false">E49*INDEX('Price List'!$Q$3:$Q$20,MATCH($C49,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E49*INDEX('Price List'!$Q$3:$Q$23,MATCH($C49,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O49" s="34" t="n">
@@ -12388,19 +12761,19 @@
         <v>16</v>
       </c>
       <c r="B50" s="16" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C50" s="32" t="s">
         <v>62</v>
       </c>
       <c r="D50" s="32" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="E50" s="33" t="n">
         <v>4</v>
       </c>
       <c r="F50" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C50,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C50,'Price List'!$C$3:$C$23,0))</f>
         <v>90800</v>
       </c>
       <c r="G50" s="20" t="n">
@@ -12408,15 +12781,15 @@
         <v>363200</v>
       </c>
       <c r="H50" s="34" t="n">
-        <f aca="false">E50*INDEX('Price List'!$K$3:$K$20,MATCH($C50,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E50*INDEX('Price List'!$K$3:$K$23,MATCH($C50,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I50" s="34" t="n">
-        <f aca="false">E50*INDEX('Price List'!$L$3:$L$20,MATCH($C50,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E50*INDEX('Price List'!$L$3:$L$23,MATCH($C50,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J50" s="34" t="n">
-        <f aca="false">E50*INDEX('Price List'!$M$3:$M$20,MATCH($C50,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E50*INDEX('Price List'!$M$3:$M$23,MATCH($C50,'Price List'!$C$3:$C$23,0))</f>
         <v>64</v>
       </c>
       <c r="K50" s="34" t="n">
@@ -12424,15 +12797,15 @@
         <v>64</v>
       </c>
       <c r="L50" s="34" t="n">
-        <f aca="false">E50*INDEX('Price List'!$O$3:$O$20,MATCH($C50,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E50*INDEX('Price List'!$O$3:$O$23,MATCH($C50,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M50" s="34" t="n">
-        <f aca="false">E50*INDEX('Price List'!$P$3:$P$20,MATCH($C50,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E50*INDEX('Price List'!$P$3:$P$23,MATCH($C50,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N50" s="34" t="n">
-        <f aca="false">E50*INDEX('Price List'!$Q$3:$Q$20,MATCH($C50,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E50*INDEX('Price List'!$Q$3:$Q$23,MATCH($C50,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O50" s="34" t="n">
@@ -12450,19 +12823,19 @@
         <v>16</v>
       </c>
       <c r="B51" s="16" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C51" s="32" t="s">
         <v>82</v>
       </c>
       <c r="D51" s="32" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E51" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F51" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C51,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C51,'Price List'!$C$3:$C$23,0))</f>
         <v>140400</v>
       </c>
       <c r="G51" s="20" t="n">
@@ -12470,15 +12843,15 @@
         <v>140400</v>
       </c>
       <c r="H51" s="34" t="n">
-        <f aca="false">E51*INDEX('Price List'!$K$3:$K$20,MATCH($C51,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E51*INDEX('Price List'!$K$3:$K$23,MATCH($C51,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I51" s="34" t="n">
-        <f aca="false">E51*INDEX('Price List'!$L$3:$L$20,MATCH($C51,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E51*INDEX('Price List'!$L$3:$L$23,MATCH($C51,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J51" s="34" t="n">
-        <f aca="false">E51*INDEX('Price List'!$M$3:$M$20,MATCH($C51,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E51*INDEX('Price List'!$M$3:$M$23,MATCH($C51,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K51" s="34" t="n">
@@ -12486,15 +12859,15 @@
         <v>0</v>
       </c>
       <c r="L51" s="34" t="n">
-        <f aca="false">E51*INDEX('Price List'!$O$3:$O$20,MATCH($C51,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E51*INDEX('Price List'!$O$3:$O$23,MATCH($C51,'Price List'!$C$3:$C$23,0))</f>
         <v>4</v>
       </c>
       <c r="M51" s="34" t="n">
-        <f aca="false">E51*INDEX('Price List'!$P$3:$P$20,MATCH($C51,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E51*INDEX('Price List'!$P$3:$P$23,MATCH($C51,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N51" s="34" t="n">
-        <f aca="false">E51*INDEX('Price List'!$Q$3:$Q$20,MATCH($C51,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E51*INDEX('Price List'!$Q$3:$Q$23,MATCH($C51,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O51" s="34" t="n">
@@ -12512,13 +12885,13 @@
         <v>16</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C52" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D52" s="36" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="E52" s="36"/>
       <c r="F52" s="36"/>
@@ -12569,19 +12942,19 @@
         <v>16</v>
       </c>
       <c r="B53" s="16" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C53" s="32" t="s">
         <v>48</v>
       </c>
       <c r="D53" s="32" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E53" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F53" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C53,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C53,'Price List'!$C$3:$C$23,0))</f>
         <v>398700</v>
       </c>
       <c r="G53" s="20" t="n">
@@ -12589,15 +12962,15 @@
         <v>398700</v>
       </c>
       <c r="H53" s="34" t="n">
-        <f aca="false">E53*INDEX('Price List'!$K$3:$K$20,MATCH($C53,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E53*INDEX('Price List'!$K$3:$K$23,MATCH($C53,'Price List'!$C$3:$C$23,0))</f>
         <v>14</v>
       </c>
       <c r="I53" s="34" t="n">
-        <f aca="false">E53*INDEX('Price List'!$L$3:$L$20,MATCH($C53,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E53*INDEX('Price List'!$L$3:$L$23,MATCH($C53,'Price List'!$C$3:$C$23,0))</f>
         <v>10</v>
       </c>
       <c r="J53" s="34" t="n">
-        <f aca="false">E53*INDEX('Price List'!$M$3:$M$20,MATCH($C53,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E53*INDEX('Price List'!$M$3:$M$23,MATCH($C53,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K53" s="34" t="n">
@@ -12605,15 +12978,15 @@
         <v>10</v>
       </c>
       <c r="L53" s="34" t="n">
-        <f aca="false">E53*INDEX('Price List'!$O$3:$O$20,MATCH($C53,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E53*INDEX('Price List'!$O$3:$O$23,MATCH($C53,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M53" s="34" t="n">
-        <f aca="false">E53*INDEX('Price List'!$P$3:$P$20,MATCH($C53,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E53*INDEX('Price List'!$P$3:$P$23,MATCH($C53,'Price List'!$C$3:$C$23,0))</f>
         <v>2</v>
       </c>
       <c r="N53" s="34" t="n">
-        <f aca="false">E53*INDEX('Price List'!$Q$3:$Q$20,MATCH($C53,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E53*INDEX('Price List'!$Q$3:$Q$23,MATCH($C53,'Price List'!$C$3:$C$23,0))</f>
         <v>1</v>
       </c>
       <c r="O53" s="34" t="n">
@@ -12631,19 +13004,19 @@
         <v>16</v>
       </c>
       <c r="B54" s="16" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C54" s="32" t="s">
         <v>58</v>
       </c>
       <c r="D54" s="32" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="E54" s="33" t="n">
         <v>6</v>
       </c>
       <c r="F54" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C54,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C54,'Price List'!$C$3:$C$23,0))</f>
         <v>91200</v>
       </c>
       <c r="G54" s="20" t="n">
@@ -12651,15 +13024,15 @@
         <v>547200</v>
       </c>
       <c r="H54" s="34" t="n">
-        <f aca="false">E54*INDEX('Price List'!$K$3:$K$20,MATCH($C54,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E54*INDEX('Price List'!$K$3:$K$23,MATCH($C54,'Price List'!$C$3:$C$23,0))</f>
         <v>96</v>
       </c>
       <c r="I54" s="34" t="n">
-        <f aca="false">E54*INDEX('Price List'!$L$3:$L$20,MATCH($C54,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E54*INDEX('Price List'!$L$3:$L$23,MATCH($C54,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J54" s="34" t="n">
-        <f aca="false">E54*INDEX('Price List'!$M$3:$M$20,MATCH($C54,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E54*INDEX('Price List'!$M$3:$M$23,MATCH($C54,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K54" s="34" t="n">
@@ -12667,15 +13040,15 @@
         <v>0</v>
       </c>
       <c r="L54" s="34" t="n">
-        <f aca="false">E54*INDEX('Price List'!$O$3:$O$20,MATCH($C54,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E54*INDEX('Price List'!$O$3:$O$23,MATCH($C54,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M54" s="34" t="n">
-        <f aca="false">E54*INDEX('Price List'!$P$3:$P$20,MATCH($C54,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E54*INDEX('Price List'!$P$3:$P$23,MATCH($C54,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N54" s="34" t="n">
-        <f aca="false">E54*INDEX('Price List'!$Q$3:$Q$20,MATCH($C54,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E54*INDEX('Price List'!$Q$3:$Q$23,MATCH($C54,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O54" s="34" t="n">
@@ -12693,19 +13066,19 @@
         <v>16</v>
       </c>
       <c r="B55" s="16" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C55" s="32" t="s">
         <v>62</v>
       </c>
       <c r="D55" s="32" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="E55" s="33" t="n">
         <v>4</v>
       </c>
       <c r="F55" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C55,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C55,'Price List'!$C$3:$C$23,0))</f>
         <v>90800</v>
       </c>
       <c r="G55" s="20" t="n">
@@ -12713,15 +13086,15 @@
         <v>363200</v>
       </c>
       <c r="H55" s="34" t="n">
-        <f aca="false">E55*INDEX('Price List'!$K$3:$K$20,MATCH($C55,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E55*INDEX('Price List'!$K$3:$K$23,MATCH($C55,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I55" s="34" t="n">
-        <f aca="false">E55*INDEX('Price List'!$L$3:$L$20,MATCH($C55,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E55*INDEX('Price List'!$L$3:$L$23,MATCH($C55,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J55" s="34" t="n">
-        <f aca="false">E55*INDEX('Price List'!$M$3:$M$20,MATCH($C55,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E55*INDEX('Price List'!$M$3:$M$23,MATCH($C55,'Price List'!$C$3:$C$23,0))</f>
         <v>64</v>
       </c>
       <c r="K55" s="34" t="n">
@@ -12729,15 +13102,15 @@
         <v>64</v>
       </c>
       <c r="L55" s="34" t="n">
-        <f aca="false">E55*INDEX('Price List'!$O$3:$O$20,MATCH($C55,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E55*INDEX('Price List'!$O$3:$O$23,MATCH($C55,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="M55" s="34" t="n">
-        <f aca="false">E55*INDEX('Price List'!$P$3:$P$20,MATCH($C55,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E55*INDEX('Price List'!$P$3:$P$23,MATCH($C55,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N55" s="34" t="n">
-        <f aca="false">E55*INDEX('Price List'!$Q$3:$Q$20,MATCH($C55,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E55*INDEX('Price List'!$Q$3:$Q$23,MATCH($C55,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O55" s="34" t="n">
@@ -12755,19 +13128,19 @@
         <v>16</v>
       </c>
       <c r="B56" s="16" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C56" s="32" t="s">
         <v>82</v>
       </c>
       <c r="D56" s="32" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E56" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F56" s="20" t="n">
-        <f aca="false">INDEX('Price List'!$I$3:$I$20,MATCH($C56,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">INDEX('Price List'!$I$3:$I$23,MATCH($C56,'Price List'!$C$3:$C$23,0))</f>
         <v>140400</v>
       </c>
       <c r="G56" s="20" t="n">
@@ -12775,15 +13148,15 @@
         <v>140400</v>
       </c>
       <c r="H56" s="34" t="n">
-        <f aca="false">E56*INDEX('Price List'!$K$3:$K$20,MATCH($C56,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E56*INDEX('Price List'!$K$3:$K$23,MATCH($C56,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="I56" s="34" t="n">
-        <f aca="false">E56*INDEX('Price List'!$L$3:$L$20,MATCH($C56,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E56*INDEX('Price List'!$L$3:$L$23,MATCH($C56,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="J56" s="34" t="n">
-        <f aca="false">E56*INDEX('Price List'!$M$3:$M$20,MATCH($C56,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E56*INDEX('Price List'!$M$3:$M$23,MATCH($C56,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="K56" s="34" t="n">
@@ -12791,15 +13164,15 @@
         <v>0</v>
       </c>
       <c r="L56" s="34" t="n">
-        <f aca="false">E56*INDEX('Price List'!$O$3:$O$20,MATCH($C56,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E56*INDEX('Price List'!$O$3:$O$23,MATCH($C56,'Price List'!$C$3:$C$23,0))</f>
         <v>4</v>
       </c>
       <c r="M56" s="34" t="n">
-        <f aca="false">E56*INDEX('Price List'!$P$3:$P$20,MATCH($C56,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E56*INDEX('Price List'!$P$3:$P$23,MATCH($C56,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="N56" s="34" t="n">
-        <f aca="false">E56*INDEX('Price List'!$Q$3:$Q$20,MATCH($C56,'Price List'!$C$3:$C$20,0))</f>
+        <f aca="false">E56*INDEX('Price List'!$Q$3:$Q$23,MATCH($C56,'Price List'!$C$3:$C$23,0))</f>
         <v>0</v>
       </c>
       <c r="O56" s="34" t="n">
@@ -12817,13 +13190,13 @@
         <v>16</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C57" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D57" s="36" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E57" s="36"/>
       <c r="F57" s="36"/>
@@ -12894,7 +13267,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -12910,7 +13283,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -12923,7 +13296,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="38" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B2" s="38"/>
       <c r="C2" s="38"/>
@@ -12942,18 +13315,18 @@
         <v>46</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="I3" s="2"/>
     </row>
@@ -12962,22 +13335,22 @@
       <c r="B4" s="15"/>
       <c r="C4" s="15"/>
       <c r="D4" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13665,55 +14038,169 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="36" t="s">
+      <c r="A23" s="39" t="str">
+        <f aca="false">'Price List'!C21</f>
+        <v>TM241CE40T</v>
+      </c>
+      <c r="B23" s="39" t="str">
+        <f aca="false">'Price List'!R21</f>
+        <v>CPU, Ethernet, 24VDC (10/06 추가 견적)</v>
+      </c>
+      <c r="C23" s="40" t="n">
+        <f aca="false">'Price List'!I21</f>
+        <v>414000</v>
+      </c>
+      <c r="D23" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A23,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="20" t="n">
+        <f aca="false">D23*$C23</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A23,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="20" t="n">
+        <f aca="false">F23*$C23</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A23,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="20" t="n">
+        <f aca="false">H23*$C23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="39" t="str">
+        <f aca="false">'Price List'!C22</f>
+        <v>TM3XTRA1</v>
+      </c>
+      <c r="B24" s="39" t="str">
+        <f aca="false">'Price List'!R22</f>
+        <v>TM3 버스 확장 송신 (10/06 추가 견적)</v>
+      </c>
+      <c r="C24" s="40" t="n">
+        <f aca="false">'Price List'!I22</f>
+        <v>62400</v>
+      </c>
+      <c r="D24" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A24,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="20" t="n">
+        <f aca="false">D24*$C24</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A24,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="20" t="n">
+        <f aca="false">F24*$C24</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A24,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="20" t="n">
+        <f aca="false">H24*$C24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="39" t="str">
+        <f aca="false">'Price List'!C23</f>
+        <v>TM3XREC1</v>
+      </c>
+      <c r="B25" s="39" t="str">
+        <f aca="false">'Price List'!R23</f>
+        <v>TM3 버스 확장 수신 (10/06 추가 견적)</v>
+      </c>
+      <c r="C25" s="40" t="n">
+        <f aca="false">'Price List'!I23</f>
+        <v>74000</v>
+      </c>
+      <c r="D25" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A25,'기준사양 매칭'!$B$5:$B$200,"A")</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="20" t="n">
+        <f aca="false">D25*$C25</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A25,'기준사양 매칭'!$B$5:$B$200,"B")</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="20" t="n">
+        <f aca="false">F25*$C25</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="20" t="n">
+        <f aca="false">SUMIFS('기준사양 매칭'!$Q$5:$Q$200,'기준사양 매칭'!$C$5:$C$200,$A25,'기준사양 매칭'!$B$5:$B$200,"C")</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="20" t="n">
+        <f aca="false">H25*$C25</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="36"/>
-      <c r="C23" s="36"/>
-      <c r="D23" s="10" t="n">
-        <f aca="false">SUM(D5:D22)</f>
+      <c r="B26" s="36"/>
+      <c r="C26" s="36"/>
+      <c r="D26" s="10" t="n">
+        <f aca="false">SUM(D5:D25)</f>
         <v>2650</v>
       </c>
-      <c r="E23" s="10" t="n">
-        <f aca="false">SUM(E5:E22)</f>
+      <c r="E26" s="10" t="n">
+        <f aca="false">SUM(E5:E25)</f>
         <v>452797500</v>
       </c>
-      <c r="F23" s="10" t="n">
-        <f aca="false">SUM(F5:F22)</f>
+      <c r="F26" s="10" t="n">
+        <f aca="false">SUM(F5:F25)</f>
         <v>2100</v>
       </c>
-      <c r="G23" s="10" t="n">
-        <f aca="false">SUM(G5:G22)</f>
+      <c r="G26" s="10" t="n">
+        <f aca="false">SUM(G5:G25)</f>
         <v>416882500</v>
       </c>
-      <c r="H23" s="10" t="n">
-        <f aca="false">SUM(H5:H22)</f>
+      <c r="H26" s="10" t="n">
+        <f aca="false">SUM(H5:H25)</f>
         <v>2100</v>
       </c>
-      <c r="I23" s="10" t="n">
-        <f aca="false">SUM(I5:I22)</f>
+      <c r="I26" s="10" t="n">
+        <f aca="false">SUM(I5:I25)</f>
         <v>411482500</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="41" t="s">
-        <v>136</v>
-      </c>
-      <c r="B24" s="41"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="42"/>
-      <c r="E24" s="42" t="str">
-        <f aca="false">IF(ABS(E23-요약!G8)&lt;1,"일치","불일치")</f>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="41" t="s">
+        <v>142</v>
+      </c>
+      <c r="B27" s="41"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="42"/>
+      <c r="E27" s="42" t="str">
+        <f aca="false">IF(ABS(E26-요약!G8)&lt;1,"일치","불일치")</f>
         <v>일치</v>
       </c>
-      <c r="F24" s="42"/>
-      <c r="G24" s="42" t="str">
-        <f aca="false">IF(ABS(G23-요약!H8)&lt;1,"일치","불일치")</f>
+      <c r="F27" s="42"/>
+      <c r="G27" s="42" t="str">
+        <f aca="false">IF(ABS(G26-요약!H8)&lt;1,"일치","불일치")</f>
         <v>일치</v>
       </c>
-      <c r="H24" s="42"/>
-      <c r="I24" s="42" t="str">
-        <f aca="false">IF(ABS(I23-요약!I8)&lt;1,"일치","불일치")</f>
+      <c r="H27" s="42"/>
+      <c r="I27" s="42" t="str">
+        <f aca="false">IF(ABS(I26-요약!I8)&lt;1,"일치","불일치")</f>
         <v>일치</v>
       </c>
     </row>
@@ -13727,8 +14214,8 @@
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="H3:I3"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A27:C27"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -13764,7 +14251,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="43" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B1" s="43"/>
       <c r="C1" s="43"/>
@@ -13783,7 +14270,7 @@
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="26" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -13802,16 +14289,16 @@
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>39</v>
@@ -13826,7 +14313,7 @@
         <v>45</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -13837,7 +14324,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>143</v>
+        <v>84</v>
       </c>
       <c r="B5" s="44" t="n">
         <v>941000</v>
@@ -13862,7 +14349,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="47" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="J5" s="47"/>
       <c r="K5" s="47"/>
@@ -13876,28 +14363,28 @@
         <v>1</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>32</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="G7" s="15" t="s">
         <v>39</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J7" s="15" t="s">
         <v>43</v>
@@ -13909,13 +14396,13 @@
         <v>45</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13923,7 +14410,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C8" s="32" t="s">
         <v>53</v>
@@ -13932,7 +14419,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C8,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C8,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C8,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C8,$A$5:$A$5,0)),0))</f>
         <v>384750</v>
       </c>
       <c r="F8" s="46" t="n">
@@ -13940,27 +14427,27 @@
         <v>384750</v>
       </c>
       <c r="G8" s="34" t="n">
-        <f aca="false">D8*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C8,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C8,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D8*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C8,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C8,$A$5:$A$5,0)),0))</f>
         <v>14</v>
       </c>
       <c r="H8" s="34" t="n">
-        <f aca="false">D8*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C8,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C8,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C8,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D8*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C8,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C8,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C8,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>10</v>
       </c>
       <c r="I8" s="34" t="n">
-        <f aca="false">D8*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C8,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D8*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C8,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>6</v>
       </c>
       <c r="J8" s="34" t="n">
-        <f aca="false">D8*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C8,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D8*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C8,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="K8" s="34" t="n">
-        <f aca="false">D8*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C8,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C8,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D8*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C8,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C8,$A$5:$A$5,0)),0))</f>
         <v>2</v>
       </c>
       <c r="L8" s="34" t="n">
-        <f aca="false">D8*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C8,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C8,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D8*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C8,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C8,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M8" s="32"/>
@@ -13972,10 +14459,10 @@
         <v>10</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C9" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D9" s="36"/>
       <c r="E9" s="36"/>
@@ -14025,7 +14512,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C11" s="32" t="s">
         <v>51</v>
@@ -14034,7 +14521,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C11,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C11,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C11,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C11,$A$5:$A$5,0)),0))</f>
         <v>392850</v>
       </c>
       <c r="F11" s="46" t="n">
@@ -14042,27 +14529,27 @@
         <v>392850</v>
       </c>
       <c r="G11" s="34" t="n">
-        <f aca="false">D11*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C11,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C11,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D11*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C11,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C11,$A$5:$A$5,0)),0))</f>
         <v>14</v>
       </c>
       <c r="H11" s="34" t="n">
-        <f aca="false">D11*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C11,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C11,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C11,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D11*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C11,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C11,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C11,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>10</v>
       </c>
       <c r="I11" s="34" t="n">
-        <f aca="false">D11*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C11,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D11*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C11,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="J11" s="34" t="n">
-        <f aca="false">D11*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C11,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D11*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C11,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="K11" s="34" t="n">
-        <f aca="false">D11*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C11,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C11,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D11*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C11,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C11,$A$5:$A$5,0)),0))</f>
         <v>2</v>
       </c>
       <c r="L11" s="34" t="n">
-        <f aca="false">D11*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C11,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C11,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D11*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C11,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C11,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M11" s="32"/>
@@ -14074,10 +14561,10 @@
         <v>10</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D12" s="36"/>
       <c r="E12" s="36"/>
@@ -14127,7 +14614,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C14" s="32" t="s">
         <v>57</v>
@@ -14136,7 +14623,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C14,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C14,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C14,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C14,$A$5:$A$5,0)),0))</f>
         <v>406350</v>
       </c>
       <c r="F14" s="46" t="n">
@@ -14144,27 +14631,27 @@
         <v>406350</v>
       </c>
       <c r="G14" s="34" t="n">
-        <f aca="false">D14*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C14,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C14,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D14*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C14,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C14,$A$5:$A$5,0)),0))</f>
         <v>24</v>
       </c>
       <c r="H14" s="34" t="n">
-        <f aca="false">D14*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C14,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C14,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C14,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D14*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C14,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C14,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C14,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>16</v>
       </c>
       <c r="I14" s="34" t="n">
-        <f aca="false">D14*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C14,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D14*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C14,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>12</v>
       </c>
       <c r="J14" s="34" t="n">
-        <f aca="false">D14*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C14,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D14*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C14,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="K14" s="34" t="n">
-        <f aca="false">D14*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C14,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C14,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D14*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C14,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C14,$A$5:$A$5,0)),0))</f>
         <v>2</v>
       </c>
       <c r="L14" s="34" t="n">
-        <f aca="false">D14*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C14,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C14,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D14*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C14,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C14,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M14" s="32"/>
@@ -14176,10 +14663,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C15" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D15" s="36"/>
       <c r="E15" s="36"/>
@@ -14229,7 +14716,7 @@
         <v>12</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C17" s="32" t="s">
         <v>56</v>
@@ -14238,7 +14725,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C17,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C17,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C17,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C17,$A$5:$A$5,0)),0))</f>
         <v>417600</v>
       </c>
       <c r="F17" s="46" t="n">
@@ -14246,27 +14733,27 @@
         <v>417600</v>
       </c>
       <c r="G17" s="34" t="n">
-        <f aca="false">D17*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C17,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C17,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D17*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C17,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C17,$A$5:$A$5,0)),0))</f>
         <v>24</v>
       </c>
       <c r="H17" s="34" t="n">
-        <f aca="false">D17*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C17,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C17,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C17,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D17*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C17,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C17,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C17,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>16</v>
       </c>
       <c r="I17" s="34" t="n">
-        <f aca="false">D17*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C17,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D17*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C17,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="J17" s="34" t="n">
-        <f aca="false">D17*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C17,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D17*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C17,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="K17" s="34" t="n">
-        <f aca="false">D17*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C17,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C17,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D17*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C17,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C17,$A$5:$A$5,0)),0))</f>
         <v>2</v>
       </c>
       <c r="L17" s="34" t="n">
-        <f aca="false">D17*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C17,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C17,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D17*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C17,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C17,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M17" s="32"/>
@@ -14278,10 +14765,10 @@
         <v>12</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C18" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D18" s="36"/>
       <c r="E18" s="36"/>
@@ -14331,7 +14818,7 @@
         <v>14</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C20" s="32" t="s">
         <v>53</v>
@@ -14340,7 +14827,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C20,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C20,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C20,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C20,$A$5:$A$5,0)),0))</f>
         <v>384750</v>
       </c>
       <c r="F20" s="46" t="n">
@@ -14348,27 +14835,27 @@
         <v>384750</v>
       </c>
       <c r="G20" s="34" t="n">
-        <f aca="false">D20*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C20,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C20,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D20*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C20,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C20,$A$5:$A$5,0)),0))</f>
         <v>14</v>
       </c>
       <c r="H20" s="34" t="n">
-        <f aca="false">D20*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C20,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C20,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C20,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D20*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C20,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C20,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C20,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>10</v>
       </c>
       <c r="I20" s="34" t="n">
-        <f aca="false">D20*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C20,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D20*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C20,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>6</v>
       </c>
       <c r="J20" s="34" t="n">
-        <f aca="false">D20*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C20,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D20*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C20,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="K20" s="34" t="n">
-        <f aca="false">D20*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C20,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C20,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D20*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C20,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C20,$A$5:$A$5,0)),0))</f>
         <v>2</v>
       </c>
       <c r="L20" s="34" t="n">
-        <f aca="false">D20*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C20,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C20,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D20*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C20,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C20,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M20" s="32"/>
@@ -14380,7 +14867,7 @@
         <v>14</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C21" s="32" t="s">
         <v>80</v>
@@ -14389,7 +14876,7 @@
         <v>1</v>
       </c>
       <c r="E21" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C21,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C21,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C21,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C21,$A$5:$A$5,0)),0))</f>
         <v>138400</v>
       </c>
       <c r="F21" s="46" t="n">
@@ -14397,27 +14884,27 @@
         <v>138400</v>
       </c>
       <c r="G21" s="34" t="n">
-        <f aca="false">D21*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C21,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C21,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D21*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C21,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C21,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="H21" s="34" t="n">
-        <f aca="false">D21*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C21,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C21,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C21,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D21*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C21,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C21,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C21,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>0</v>
       </c>
       <c r="I21" s="34" t="n">
-        <f aca="false">D21*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C21,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D21*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C21,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="J21" s="34" t="n">
-        <f aca="false">D21*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C21,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D21*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C21,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>2</v>
       </c>
       <c r="K21" s="34" t="n">
-        <f aca="false">D21*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C21,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C21,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D21*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C21,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C21,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="L21" s="34" t="n">
-        <f aca="false">D21*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C21,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C21,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D21*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C21,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C21,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M21" s="32"/>
@@ -14429,10 +14916,10 @@
         <v>14</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C22" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D22" s="36"/>
       <c r="E22" s="36"/>
@@ -14482,7 +14969,7 @@
         <v>14</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C24" s="32" t="s">
         <v>51</v>
@@ -14491,7 +14978,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C24,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C24,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C24,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C24,$A$5:$A$5,0)),0))</f>
         <v>392850</v>
       </c>
       <c r="F24" s="46" t="n">
@@ -14499,27 +14986,27 @@
         <v>392850</v>
       </c>
       <c r="G24" s="34" t="n">
-        <f aca="false">D24*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C24,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C24,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D24*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C24,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C24,$A$5:$A$5,0)),0))</f>
         <v>14</v>
       </c>
       <c r="H24" s="34" t="n">
-        <f aca="false">D24*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C24,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C24,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C24,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D24*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C24,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C24,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C24,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>10</v>
       </c>
       <c r="I24" s="34" t="n">
-        <f aca="false">D24*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C24,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D24*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C24,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="J24" s="34" t="n">
-        <f aca="false">D24*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C24,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D24*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C24,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="K24" s="34" t="n">
-        <f aca="false">D24*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C24,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C24,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D24*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C24,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C24,$A$5:$A$5,0)),0))</f>
         <v>2</v>
       </c>
       <c r="L24" s="34" t="n">
-        <f aca="false">D24*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C24,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C24,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D24*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C24,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C24,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M24" s="32"/>
@@ -14531,7 +15018,7 @@
         <v>14</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C25" s="32" t="s">
         <v>80</v>
@@ -14540,7 +15027,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C25,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C25,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C25,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C25,$A$5:$A$5,0)),0))</f>
         <v>138400</v>
       </c>
       <c r="F25" s="46" t="n">
@@ -14548,27 +15035,27 @@
         <v>138400</v>
       </c>
       <c r="G25" s="34" t="n">
-        <f aca="false">D25*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C25,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C25,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D25*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C25,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C25,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="H25" s="34" t="n">
-        <f aca="false">D25*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C25,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C25,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C25,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D25*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C25,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C25,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C25,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>0</v>
       </c>
       <c r="I25" s="34" t="n">
-        <f aca="false">D25*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C25,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D25*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C25,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="J25" s="34" t="n">
-        <f aca="false">D25*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C25,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D25*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C25,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>2</v>
       </c>
       <c r="K25" s="34" t="n">
-        <f aca="false">D25*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C25,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C25,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D25*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C25,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C25,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="L25" s="34" t="n">
-        <f aca="false">D25*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C25,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C25,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D25*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C25,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C25,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M25" s="32"/>
@@ -14580,10 +15067,10 @@
         <v>14</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C26" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D26" s="36"/>
       <c r="E26" s="36"/>
@@ -14633,44 +15120,44 @@
         <v>16</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C28" s="32" t="s">
-        <v>143</v>
+        <v>84</v>
       </c>
       <c r="D28" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="50" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C28,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C28,$A$5:$A$5,0)),0))</f>
-        <v>423450</v>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C28,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C28,$A$5:$A$5,0)),0))</f>
+        <v>414000</v>
       </c>
       <c r="F28" s="46" t="n">
         <f aca="false">D28*E28</f>
-        <v>423450</v>
+        <v>414000</v>
       </c>
       <c r="G28" s="34" t="n">
-        <f aca="false">D28*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C28,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C28,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D28*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C28,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C28,$A$5:$A$5,0)),0))</f>
         <v>24</v>
       </c>
       <c r="H28" s="34" t="n">
-        <f aca="false">D28*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C28,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C28,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C28,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D28*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C28,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C28,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C28,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>16</v>
       </c>
       <c r="I28" s="34" t="n">
-        <f aca="false">D28*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C28,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D28*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C28,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="J28" s="34" t="n">
-        <f aca="false">D28*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C28,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D28*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C28,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="K28" s="34" t="n">
-        <f aca="false">D28*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C28,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C28,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D28*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C28,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C28,$A$5:$A$5,0)),0))</f>
         <v>2</v>
       </c>
       <c r="L28" s="34" t="n">
-        <f aca="false">D28*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C28,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C28,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D28*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C28,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C28,$A$5:$A$5,0)),0))</f>
         <v>1</v>
       </c>
       <c r="M28" s="32"/>
@@ -14682,7 +15169,7 @@
         <v>16</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C29" s="32" t="s">
         <v>58</v>
@@ -14691,7 +15178,7 @@
         <v>2</v>
       </c>
       <c r="E29" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C29,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C29,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C29,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C29,$A$5:$A$5,0)),0))</f>
         <v>91200</v>
       </c>
       <c r="F29" s="46" t="n">
@@ -14699,27 +15186,27 @@
         <v>182400</v>
       </c>
       <c r="G29" s="34" t="n">
-        <f aca="false">D29*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C29,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C29,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D29*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C29,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C29,$A$5:$A$5,0)),0))</f>
         <v>32</v>
       </c>
       <c r="H29" s="34" t="n">
-        <f aca="false">D29*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C29,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C29,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C29,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D29*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C29,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C29,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C29,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>0</v>
       </c>
       <c r="I29" s="34" t="n">
-        <f aca="false">D29*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C29,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D29*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C29,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="J29" s="34" t="n">
-        <f aca="false">D29*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C29,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D29*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C29,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="K29" s="34" t="n">
-        <f aca="false">D29*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C29,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C29,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D29*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C29,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C29,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="L29" s="34" t="n">
-        <f aca="false">D29*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C29,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C29,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D29*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C29,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C29,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M29" s="32"/>
@@ -14731,7 +15218,7 @@
         <v>16</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C30" s="32" t="s">
         <v>60</v>
@@ -14740,7 +15227,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C30,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C30,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C30,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C30,$A$5:$A$5,0)),0))</f>
         <v>80800</v>
       </c>
       <c r="F30" s="46" t="n">
@@ -14748,27 +15235,27 @@
         <v>80800</v>
       </c>
       <c r="G30" s="34" t="n">
-        <f aca="false">D30*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C30,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C30,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D30*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C30,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C30,$A$5:$A$5,0)),0))</f>
         <v>8</v>
       </c>
       <c r="H30" s="34" t="n">
-        <f aca="false">D30*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C30,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C30,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C30,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D30*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C30,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C30,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C30,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>0</v>
       </c>
       <c r="I30" s="34" t="n">
-        <f aca="false">D30*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C30,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D30*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C30,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="J30" s="34" t="n">
-        <f aca="false">D30*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C30,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D30*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C30,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="K30" s="34" t="n">
-        <f aca="false">D30*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C30,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C30,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D30*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C30,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C30,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="L30" s="34" t="n">
-        <f aca="false">D30*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C30,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C30,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D30*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C30,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C30,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M30" s="32"/>
@@ -14780,7 +15267,7 @@
         <v>16</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C31" s="32" t="s">
         <v>64</v>
@@ -14789,7 +15276,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C31,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C31,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C31,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C31,$A$5:$A$5,0)),0))</f>
         <v>90800</v>
       </c>
       <c r="F31" s="46" t="n">
@@ -14797,27 +15284,27 @@
         <v>90800</v>
       </c>
       <c r="G31" s="34" t="n">
-        <f aca="false">D31*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C31,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C31,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D31*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C31,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C31,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="H31" s="34" t="n">
-        <f aca="false">D31*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C31,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C31,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C31,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D31*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C31,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C31,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C31,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>16</v>
       </c>
       <c r="I31" s="34" t="n">
-        <f aca="false">D31*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C31,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D31*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C31,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="J31" s="34" t="n">
-        <f aca="false">D31*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C31,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D31*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C31,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="K31" s="34" t="n">
-        <f aca="false">D31*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C31,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C31,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D31*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C31,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C31,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="L31" s="34" t="n">
-        <f aca="false">D31*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C31,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C31,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D31*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C31,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C31,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M31" s="32"/>
@@ -14829,7 +15316,7 @@
         <v>16</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C32" s="32" t="s">
         <v>70</v>
@@ -14838,7 +15325,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C32,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C32,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C32,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C32,$A$5:$A$5,0)),0))</f>
         <v>67200</v>
       </c>
       <c r="F32" s="46" t="n">
@@ -14846,27 +15333,27 @@
         <v>67200</v>
       </c>
       <c r="G32" s="34" t="n">
-        <f aca="false">D32*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C32,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C32,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D32*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C32,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C32,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="H32" s="34" t="n">
-        <f aca="false">D32*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C32,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C32,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C32,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D32*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C32,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C32,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C32,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>8</v>
       </c>
       <c r="I32" s="34" t="n">
-        <f aca="false">D32*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C32,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D32*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C32,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="J32" s="34" t="n">
-        <f aca="false">D32*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C32,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D32*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C32,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="K32" s="34" t="n">
-        <f aca="false">D32*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C32,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C32,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D32*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C32,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C32,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="L32" s="34" t="n">
-        <f aca="false">D32*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C32,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C32,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D32*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C32,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C32,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M32" s="32"/>
@@ -14878,7 +15365,7 @@
         <v>16</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C33" s="32" t="s">
         <v>80</v>
@@ -14887,7 +15374,7 @@
         <v>1</v>
       </c>
       <c r="E33" s="46" t="n">
-        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$20,MATCH($C33,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C33,$A$5:$A$5,0)),0))</f>
+        <f aca="false">IFERROR(INDEX('Price List'!$I$3:$I$23,MATCH($C33,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($D$5:$D$5,MATCH($C33,$A$5:$A$5,0)),0))</f>
         <v>138400</v>
       </c>
       <c r="F33" s="46" t="n">
@@ -14895,27 +15382,27 @@
         <v>138400</v>
       </c>
       <c r="G33" s="34" t="n">
-        <f aca="false">D33*IFERROR(INDEX('Price List'!$K$3:$K$20,MATCH($C33,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C33,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D33*IFERROR(INDEX('Price List'!$K$3:$K$23,MATCH($C33,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($E$5:$E$5,MATCH($C33,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="H33" s="34" t="n">
-        <f aca="false">D33*(IFERROR(INDEX('Price List'!$L$3:$L$20,MATCH($C33,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C33,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C33,'Price List'!$C$3:$C$20,0)),0))</f>
+        <f aca="false">D33*(IFERROR(INDEX('Price List'!$L$3:$L$23,MATCH($C33,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($F$5:$F$5,MATCH($C33,$A$5:$A$5,0)),0))+IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C33,'Price List'!$C$3:$C$23,0)),0))</f>
         <v>0</v>
       </c>
       <c r="I33" s="34" t="n">
-        <f aca="false">D33*IFERROR(INDEX('Price List'!$M$3:$M$20,MATCH($C33,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D33*IFERROR(INDEX('Price List'!$M$3:$M$23,MATCH($C33,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>0</v>
       </c>
       <c r="J33" s="34" t="n">
-        <f aca="false">D33*IFERROR(INDEX('Price List'!$O$3:$O$20,MATCH($C33,'Price List'!$C$3:$C$20,0)),0)</f>
+        <f aca="false">D33*IFERROR(INDEX('Price List'!$O$3:$O$23,MATCH($C33,'Price List'!$C$3:$C$23,0)),0)</f>
         <v>2</v>
       </c>
       <c r="K33" s="34" t="n">
-        <f aca="false">D33*IFERROR(INDEX('Price List'!$P$3:$P$20,MATCH($C33,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C33,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D33*IFERROR(INDEX('Price List'!$P$3:$P$23,MATCH($C33,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($G$5:$G$5,MATCH($C33,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="L33" s="34" t="n">
-        <f aca="false">D33*IFERROR(INDEX('Price List'!$Q$3:$Q$20,MATCH($C33,'Price List'!$C$3:$C$20,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C33,$A$5:$A$5,0)),0))</f>
+        <f aca="false">D33*IFERROR(INDEX('Price List'!$Q$3:$Q$23,MATCH($C33,'Price List'!$C$3:$C$23,0)),IFERROR(INDEX($H$5:$H$5,MATCH($C33,$A$5:$A$5,0)),0))</f>
         <v>0</v>
       </c>
       <c r="M33" s="32"/>
@@ -14927,16 +15414,16 @@
         <v>16</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C34" s="36" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D34" s="36"/>
       <c r="E34" s="36"/>
       <c r="F34" s="48" t="n">
         <f aca="false">SUM(F28:F33)</f>
-        <v>983050</v>
+        <v>973600</v>
       </c>
       <c r="G34" s="37" t="n">
         <f aca="false">SUM(G28:G33)</f>
@@ -14968,7 +15455,7 @@
       </c>
       <c r="N34" s="48" t="n">
         <f aca="false">F34*M34</f>
-        <v>98305000</v>
+        <v>97360000</v>
       </c>
       <c r="O34" s="51" t="str">
         <f aca="false">IF(AND(G34&gt;='기준사양 매칭'!H42,H34&gt;='기준사양 매칭'!K42,I34&gt;='기준사양 매칭'!K42,J34&gt;='기준사양 매칭'!L42,K34&gt;='기준사양 매칭'!M42,L34&gt;='기준사양 매칭'!N42),"충족",IF(G34&lt;'기준사양 매칭'!H42,"DI "&amp;('기준사양 매칭'!H42-G34)&amp;" 부족  ","")&amp;IF(H34&lt;'기준사양 매칭'!K42,"DO "&amp;('기준사양 매칭'!K42-H34)&amp;" 부족  ","")&amp;IF(I34&lt;'기준사양 매칭'!K42,"Relay DO "&amp;('기준사양 매칭'!K42-I34)&amp;" 부족  ","")&amp;IF(J34&lt;'기준사양 매칭'!L42,"AO "&amp;('기준사양 매칭'!L42-J34)&amp;" 부족  ","")&amp;IF(K34&lt;'기준사양 매칭'!M42,"Serial "&amp;('기준사양 매칭'!M42-K34)&amp;" 부족  ","")&amp;IF(L34&lt;'기준사양 매칭'!N42,"ETH "&amp;('기준사양 매칭'!N42-L34)&amp;" 부족  ",""))</f>
@@ -14977,7 +15464,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="52" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14985,22 +15472,22 @@
         <v>1</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="E37" s="15" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="F37" s="15" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15100,11 +15587,11 @@
       </c>
       <c r="C41" s="20" t="n">
         <f aca="false">N34</f>
-        <v>98305000</v>
+        <v>97360000</v>
       </c>
       <c r="D41" s="20" t="n">
         <f aca="false">N34</f>
-        <v>98305000</v>
+        <v>97360000</v>
       </c>
       <c r="E41" s="40" t="n">
         <f aca="false">요약!H7</f>
@@ -15116,7 +15603,7 @@
       </c>
       <c r="G41" s="20" t="n">
         <f aca="false">C41-E41</f>
-        <v>-46645000</v>
+        <v>-47590000</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15129,11 +15616,11 @@
       </c>
       <c r="C42" s="10" t="n">
         <f aca="false">SUM(C38:C41)</f>
-        <v>328717500</v>
+        <v>327772500</v>
       </c>
       <c r="D42" s="10" t="n">
         <f aca="false">SUM(D38:D41)</f>
-        <v>323317500</v>
+        <v>322372500</v>
       </c>
       <c r="E42" s="10" t="n">
         <f aca="false">SUM(E38:E41)</f>
@@ -15145,12 +15632,12 @@
       </c>
       <c r="G42" s="10" t="n">
         <f aca="false">SUM(G38:G41)</f>
-        <v>-88165000</v>
+        <v>-89110000</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="55" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B43" s="55"/>
       <c r="C43" s="55"/>
@@ -15169,7 +15656,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="56" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B45" s="56"/>
       <c r="C45" s="56"/>
@@ -15188,7 +15675,7 @@
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="57" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B46" s="57"/>
       <c r="C46" s="57"/>
@@ -15207,7 +15694,7 @@
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="57" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B47" s="57"/>
       <c r="C47" s="57"/>
@@ -15226,7 +15713,7 @@
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="58" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B48" s="58"/>
       <c r="C48" s="58"/>
@@ -15245,7 +15732,7 @@
     </row>
     <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="58" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B49" s="58"/>
       <c r="C49" s="58"/>
@@ -15264,7 +15751,7 @@
     </row>
     <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="58" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B50" s="58"/>
       <c r="C50" s="58"/>
@@ -15283,7 +15770,7 @@
     </row>
     <row r="51" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="58" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B51" s="58"/>
       <c r="C51" s="58"/>
@@ -15302,7 +15789,7 @@
     </row>
     <row r="52" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="58" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="B52" s="58"/>
       <c r="C52" s="58"/>
@@ -15366,7 +15853,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="43" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B1" s="43"/>
       <c r="C1" s="43"/>
@@ -15380,7 +15867,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="59" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B3" s="60" t="n">
         <v>0.45</v>
@@ -15388,45 +15875,45 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="59" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B4" s="60" t="n">
         <v>0.4</v>
       </c>
       <c r="C4" s="61" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15706,7 +16193,7 @@
     </row>
     <row r="15" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="69" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B15" s="69"/>
       <c r="C15" s="69"/>
@@ -15720,7 +16207,7 @@
     </row>
     <row r="16" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="69" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B16" s="69"/>
       <c r="C16" s="69"/>
@@ -15734,7 +16221,7 @@
     </row>
     <row r="17" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="70" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B17" s="70"/>
       <c r="C17" s="70"/>

</xml_diff>